<commit_message>
feat: use standard English filenames for handouts on GitHub Pages
</commit_message>
<xml_diff>
--- a/文意新8課_GitHub部署檔案清單與網址對照表.xlsx
+++ b/文意新8課_GitHub部署檔案清單與網址對照表.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="已上線部署教材清單" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="全書37單元架構總表" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="已上線部署教材清單" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="全書37單元架構總表" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -575,8 +575,8 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L12"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
+  <dimension ref="A1:L18"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
     <col width="16" customWidth="1" min="2" max="2"/>
@@ -1146,6 +1146,186 @@
       <c r="L12" s="13" t="inlineStr">
         <is>
           <t>Markdown 格式排版、直覺導覽與章節超連結</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="n">
+        <v>9</v>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>第 1 課 主旨篇</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>記敘文類講義</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>01_主旨篇_記敘文類_詳解講義.pdf</t>
+        </is>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>01_main_idea_narrative_handout.pdf</t>
+        </is>
+      </c>
+      <c r="F13" t="inlineStr">
+        <is>
+          <t>https://oaoadna-1313.github.io/2026-literarymeaning8lesson/01_main_idea_narrative_handout.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="n">
+        <v>10</v>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>第 1 課 主旨篇</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>抒情文類講義</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>02_主旨篇_抒情文類_詳解講義.pdf</t>
+        </is>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>02_main_idea_lyric_handout.pdf</t>
+        </is>
+      </c>
+      <c r="F14" t="inlineStr">
+        <is>
+          <t>https://oaoadna-1313.github.io/2026-literarymeaning8lesson/02_main_idea_lyric_handout.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="n">
+        <v>11</v>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>第 1 課 主旨篇</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>議論文類講義</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>03_主旨篇_議論文類_詳解講義.pdf</t>
+        </is>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>03_main_idea_argumentative_handout.pdf</t>
+        </is>
+      </c>
+      <c r="F15" t="inlineStr">
+        <is>
+          <t>https://oaoadna-1313.github.io/2026-literarymeaning8lesson/03_main_idea_argumentative_handout.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="n">
+        <v>12</v>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>第 1 課 主旨篇</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>說明文類講義</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>04_主旨篇_說明文類_詳解講義.pdf</t>
+        </is>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>04_main_idea_expository_handout.pdf</t>
+        </is>
+      </c>
+      <c r="F16" t="inlineStr">
+        <is>
+          <t>https://oaoadna-1313.github.io/2026-literarymeaning8lesson/04_main_idea_expository_handout.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="n">
+        <v>13</v>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>第 1 課 主旨篇</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>應用文類講義</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>05_主旨篇_應用文類_詳解講義.pdf</t>
+        </is>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>05_main_idea_practical_handout.pdf</t>
+        </is>
+      </c>
+      <c r="F17" t="inlineStr">
+        <is>
+          <t>https://oaoadna-1313.github.io/2026-literarymeaning8lesson/05_main_idea_practical_handout.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="n">
+        <v>14</v>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>第 1 課 主旨篇</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>全套合訂本講義</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>文意新8課_第1課主旨篇_全套精編詳解講義.pdf</t>
+        </is>
+      </c>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>01_main_idea_complete_handout.pdf</t>
+        </is>
+      </c>
+      <c r="F18" t="inlineStr">
+        <is>
+          <t>https://oaoadna-1313.github.io/2026-literarymeaning8lesson/01_main_idea_complete_handout.pdf</t>
         </is>
       </c>
     </row>
@@ -1179,7 +1359,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:J41"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
     <col width="12" customWidth="1" min="2" max="2"/>
@@ -1207,7 +1387,6 @@
         </is>
       </c>
     </row>
-    <row r="3"/>
     <row r="4" ht="28" customHeight="1">
       <c r="A4" s="20" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
feat: deploy Lesson 02 (Viewpoint) interactive courseware, A4 handouts, complete collection PDF, and updated index
</commit_message>
<xml_diff>
--- a/文意新8課_GitHub部署檔案清單與網址對照表.xlsx
+++ b/文意新8課_GitHub部署檔案清單與網址對照表.xlsx
@@ -575,7 +575,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L18"/>
+  <dimension ref="A1:L29"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -1326,6 +1326,666 @@
       <c r="F18" t="inlineStr">
         <is>
           <t>https://oaoadna-1313.github.io/2026-literarymeaning8lesson/01_main_idea_complete_handout.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="n">
+        <v>15</v>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>第 2 課 觀點篇</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>記敘文類</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>06_觀點篇_記敘文類.html</t>
+        </is>
+      </c>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>06_viewpoint_narrative.html</t>
+        </is>
+      </c>
+      <c r="F19" t="inlineStr">
+        <is>
+          <t>P.28 ~ P.30</t>
+        </is>
+      </c>
+      <c r="G19" t="inlineStr">
+        <is>
+          <t>10 題</t>
+        </is>
+      </c>
+      <c r="H19" t="inlineStr">
+        <is>
+          <t>記敘文敘事觀點與人物心理剖析。選文包含：李白、白居易、韓非子、列子寓言、明清名篇等，掌握作者敘事視角、寓意寄託與情節深意。</t>
+        </is>
+      </c>
+      <c r="I19" t="inlineStr">
+        <is>
+          <t>https://oaoadna-1313.github.io/2026-literarymeaning8lesson/06_viewpoint_narrative.html</t>
+        </is>
+      </c>
+      <c r="J19" t="inlineStr">
+        <is>
+          <t>https://github.com/oaoadna-1313/2026-literarymeaning8lesson/blob/main/06_viewpoint_narrative.html</t>
+        </is>
+      </c>
+      <c r="K19" t="inlineStr">
+        <is>
+          <t>🟢 已就緒上線</t>
+        </is>
+      </c>
+      <c r="L19" t="inlineStr">
+        <is>
+          <t>純題模式、即時答題回饋、多色螢光筆文本高亮、逐選項深度剖析、字級縮放</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="n">
+        <v>16</v>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>第 2 課 觀點篇</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>抒情文類</t>
+        </is>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>07_觀點篇_抒情文類.html</t>
+        </is>
+      </c>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>07_viewpoint_lyric.html</t>
+        </is>
+      </c>
+      <c r="F20" t="inlineStr">
+        <is>
+          <t>P.31 ~ P.33</t>
+        </is>
+      </c>
+      <c r="G20" t="inlineStr">
+        <is>
+          <t>10 題</t>
+        </is>
+      </c>
+      <c r="H20" t="inlineStr">
+        <is>
+          <t>抒情文觀點與作者情志感知。選文包含：蘇軾、辛棄疾、古典名家詩詞與現代抒情散文，體察字裡行間的情感寄託與生命觀照。</t>
+        </is>
+      </c>
+      <c r="I20" t="inlineStr">
+        <is>
+          <t>https://oaoadna-1313.github.io/2026-literarymeaning8lesson/07_viewpoint_lyric.html</t>
+        </is>
+      </c>
+      <c r="J20" t="inlineStr">
+        <is>
+          <t>https://github.com/oaoadna-1313/2026-literarymeaning8lesson/blob/main/07_viewpoint_lyric.html</t>
+        </is>
+      </c>
+      <c r="K20" t="inlineStr">
+        <is>
+          <t>🟢 已就緒上線</t>
+        </is>
+      </c>
+      <c r="L20" t="inlineStr">
+        <is>
+          <t>純題模式、即時答題回饋、情意核心高亮標註、完整語譯與注釋、錯題記錄</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="n">
+        <v>17</v>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>第 2 課 觀點篇</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>議論文類</t>
+        </is>
+      </c>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>08_觀點篇_議論文類.html</t>
+        </is>
+      </c>
+      <c r="E21" t="inlineStr">
+        <is>
+          <t>08_viewpoint_argumentative.html</t>
+        </is>
+      </c>
+      <c r="F21" t="inlineStr">
+        <is>
+          <t>P.34 ~ P.36</t>
+        </is>
+      </c>
+      <c r="G21" t="inlineStr">
+        <is>
+          <t>10 題</t>
+        </is>
+      </c>
+      <c r="H21" t="inlineStr">
+        <is>
+          <t>議論文作者主張、立場與批判性思考。深入剖析韓愈、荀子、論語與現代論述散文，辨析論點論據邏輯與隱含價值觀。</t>
+        </is>
+      </c>
+      <c r="I21" t="inlineStr">
+        <is>
+          <t>https://oaoadna-1313.github.io/2026-literarymeaning8lesson/08_viewpoint_argumentative.html</t>
+        </is>
+      </c>
+      <c r="J21" t="inlineStr">
+        <is>
+          <t>https://github.com/oaoadna-1313/2026-literarymeaning8lesson/blob/main/08_viewpoint_argumentative.html</t>
+        </is>
+      </c>
+      <c r="K21" t="inlineStr">
+        <is>
+          <t>🟢 已就緒上線</t>
+        </is>
+      </c>
+      <c r="L21" t="inlineStr">
+        <is>
+          <t>解題之眼關鍵線索、論點句子動態螢光筆定位、逐項正誤解析、題號快速導覽</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="n">
+        <v>18</v>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>第 2 課 觀點篇</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>說明文類</t>
+        </is>
+      </c>
+      <c r="D22" t="inlineStr">
+        <is>
+          <t>09_觀點篇_說明文類.html</t>
+        </is>
+      </c>
+      <c r="E22" t="inlineStr">
+        <is>
+          <t>09_viewpoint_expository.html</t>
+        </is>
+      </c>
+      <c r="F22" t="inlineStr">
+        <is>
+          <t>P.37 ~ P.39</t>
+        </is>
+      </c>
+      <c r="G22" t="inlineStr">
+        <is>
+          <t>10 題</t>
+        </is>
+      </c>
+      <c r="H22" t="inlineStr">
+        <is>
+          <t>說明文客觀解說角度與作者視點。剖析自然科學、地理歷史、文化工藝說明文本，掌握作者說明的立足點與資訊層次。</t>
+        </is>
+      </c>
+      <c r="I22" t="inlineStr">
+        <is>
+          <t>https://oaoadna-1313.github.io/2026-literarymeaning8lesson/09_viewpoint_expository.html</t>
+        </is>
+      </c>
+      <c r="J22" t="inlineStr">
+        <is>
+          <t>https://github.com/oaoadna-1313/2026-literarymeaning8lesson/blob/main/09_viewpoint_expository.html</t>
+        </is>
+      </c>
+      <c r="K22" t="inlineStr">
+        <is>
+          <t>🟢 已就緒上線</t>
+        </is>
+      </c>
+      <c r="L22" t="inlineStr">
+        <is>
+          <t>科技科普條理標註、文本知識架構拆解、互動單題/連續切換模式</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="n">
+        <v>19</v>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>第 2 課 觀點篇</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>應用文類</t>
+        </is>
+      </c>
+      <c r="D23" t="inlineStr">
+        <is>
+          <t>10_觀點篇_應用文類.html</t>
+        </is>
+      </c>
+      <c r="E23" t="inlineStr">
+        <is>
+          <t>10_viewpoint_practical.html</t>
+        </is>
+      </c>
+      <c r="F23" t="inlineStr">
+        <is>
+          <t>P.40 ~ P.42</t>
+        </is>
+      </c>
+      <c r="G23" t="inlineStr">
+        <is>
+          <t>10 題</t>
+        </is>
+      </c>
+      <c r="H23" t="inlineStr">
+        <is>
+          <t>應用文溝通意圖、宣傳視角與生活資訊整合。解析公告啟事、各類文宣、題辭聯對與表格規章中的作者或發布者觀點立場。</t>
+        </is>
+      </c>
+      <c r="I23" t="inlineStr">
+        <is>
+          <t>https://oaoadna-1313.github.io/2026-literarymeaning8lesson/10_viewpoint_practical.html</t>
+        </is>
+      </c>
+      <c r="J23" t="inlineStr">
+        <is>
+          <t>https://github.com/oaoadna-1313/2026-literarymeaning8lesson/blob/main/10_viewpoint_practical.html</t>
+        </is>
+      </c>
+      <c r="K23" t="inlineStr">
+        <is>
+          <t>🟢 已就緒上線</t>
+        </is>
+      </c>
+      <c r="L23" t="inlineStr">
+        <is>
+          <t>情境模擬文本、圖文閱讀重點對應高亮、生活素養題組深度解構</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="n">
+        <v>20</v>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>第 2 課 觀點篇</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>記敘文類講義</t>
+        </is>
+      </c>
+      <c r="D24" t="inlineStr">
+        <is>
+          <t>06_觀點篇_記敘文類_詳解講義.pdf</t>
+        </is>
+      </c>
+      <c r="E24" t="inlineStr">
+        <is>
+          <t>06_viewpoint_narrative_handout.pdf</t>
+        </is>
+      </c>
+      <c r="F24" t="inlineStr">
+        <is>
+          <t>P.28 ~ P.30</t>
+        </is>
+      </c>
+      <c r="G24" t="inlineStr">
+        <is>
+          <t>10 頁 (10題)</t>
+        </is>
+      </c>
+      <c r="H24" t="inlineStr">
+        <is>
+          <t>A4 單元精編詳解講義。含三色擬真螢光筆脈絡標註、解題之眼直擊死穴、白話語譯與逐項剖析。</t>
+        </is>
+      </c>
+      <c r="I24" t="inlineStr">
+        <is>
+          <t>https://oaoadna-1313.github.io/2026-literarymeaning8lesson/06_viewpoint_narrative_handout.pdf</t>
+        </is>
+      </c>
+      <c r="J24" t="inlineStr">
+        <is>
+          <t>https://github.com/oaoadna-1313/2026-literarymeaning8lesson/blob/main/06_viewpoint_narrative_handout.pdf</t>
+        </is>
+      </c>
+      <c r="K24" t="inlineStr">
+        <is>
+          <t>🟢 已就緒上線</t>
+        </is>
+      </c>
+      <c r="L24" t="inlineStr">
+        <is>
+          <t>A4 向量精編、一頁一題無縫排版、三色螢光筆印刷相容</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="n">
+        <v>21</v>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>第 2 課 觀點篇</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>抒情文類講義</t>
+        </is>
+      </c>
+      <c r="D25" t="inlineStr">
+        <is>
+          <t>07_觀點篇_抒情文類_詳解講義.pdf</t>
+        </is>
+      </c>
+      <c r="E25" t="inlineStr">
+        <is>
+          <t>07_viewpoint_lyric_handout.pdf</t>
+        </is>
+      </c>
+      <c r="F25" t="inlineStr">
+        <is>
+          <t>P.31 ~ P.33</t>
+        </is>
+      </c>
+      <c r="G25" t="inlineStr">
+        <is>
+          <t>10 頁 (10題)</t>
+        </is>
+      </c>
+      <c r="H25" t="inlineStr">
+        <is>
+          <t>A4 單元精編詳解講義。含三色擬真螢光筆脈絡標註、解題之眼直擊死穴、白話語譯與逐項剖析。</t>
+        </is>
+      </c>
+      <c r="I25" t="inlineStr">
+        <is>
+          <t>https://oaoadna-1313.github.io/2026-literarymeaning8lesson/07_viewpoint_lyric_handout.pdf</t>
+        </is>
+      </c>
+      <c r="J25" t="inlineStr">
+        <is>
+          <t>https://github.com/oaoadna-1313/2026-literarymeaning8lesson/blob/main/07_viewpoint_lyric_handout.pdf</t>
+        </is>
+      </c>
+      <c r="K25" t="inlineStr">
+        <is>
+          <t>🟢 已就緒上線</t>
+        </is>
+      </c>
+      <c r="L25" t="inlineStr">
+        <is>
+          <t>A4 向量精編、一頁一題無縫排版、三色螢光筆印刷相容</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="n">
+        <v>22</v>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>第 2 課 觀點篇</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>議論文類講義</t>
+        </is>
+      </c>
+      <c r="D26" t="inlineStr">
+        <is>
+          <t>08_觀點篇_議論文類_詳解講義.pdf</t>
+        </is>
+      </c>
+      <c r="E26" t="inlineStr">
+        <is>
+          <t>08_viewpoint_argumentative_handout.pdf</t>
+        </is>
+      </c>
+      <c r="F26" t="inlineStr">
+        <is>
+          <t>P.34 ~ P.36</t>
+        </is>
+      </c>
+      <c r="G26" t="inlineStr">
+        <is>
+          <t>10 頁 (10題)</t>
+        </is>
+      </c>
+      <c r="H26" t="inlineStr">
+        <is>
+          <t>A4 單元精編詳解講義。含三色擬真螢光筆脈絡標註、解題之眼直擊死穴、白話語譯與逐項剖析。</t>
+        </is>
+      </c>
+      <c r="I26" t="inlineStr">
+        <is>
+          <t>https://oaoadna-1313.github.io/2026-literarymeaning8lesson/08_viewpoint_argumentative_handout.pdf</t>
+        </is>
+      </c>
+      <c r="J26" t="inlineStr">
+        <is>
+          <t>https://github.com/oaoadna-1313/2026-literarymeaning8lesson/blob/main/08_viewpoint_argumentative_handout.pdf</t>
+        </is>
+      </c>
+      <c r="K26" t="inlineStr">
+        <is>
+          <t>🟢 已就緒上線</t>
+        </is>
+      </c>
+      <c r="L26" t="inlineStr">
+        <is>
+          <t>A4 向量精編、一頁一題無縫排版、三色螢光筆印刷相容</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="n">
+        <v>23</v>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>第 2 課 觀點篇</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>說明文類講義</t>
+        </is>
+      </c>
+      <c r="D27" t="inlineStr">
+        <is>
+          <t>09_觀點篇_說明文類_詳解講義.pdf</t>
+        </is>
+      </c>
+      <c r="E27" t="inlineStr">
+        <is>
+          <t>09_viewpoint_expository_handout.pdf</t>
+        </is>
+      </c>
+      <c r="F27" t="inlineStr">
+        <is>
+          <t>P.37 ~ P.39</t>
+        </is>
+      </c>
+      <c r="G27" t="inlineStr">
+        <is>
+          <t>10 頁 (10題)</t>
+        </is>
+      </c>
+      <c r="H27" t="inlineStr">
+        <is>
+          <t>A4 單元精編詳解講義。含三色擬真螢光筆脈絡標註、解題之眼直擊死穴、白話語譯與逐項剖析。</t>
+        </is>
+      </c>
+      <c r="I27" t="inlineStr">
+        <is>
+          <t>https://oaoadna-1313.github.io/2026-literarymeaning8lesson/09_viewpoint_expository_handout.pdf</t>
+        </is>
+      </c>
+      <c r="J27" t="inlineStr">
+        <is>
+          <t>https://github.com/oaoadna-1313/2026-literarymeaning8lesson/blob/main/09_viewpoint_expository_handout.pdf</t>
+        </is>
+      </c>
+      <c r="K27" t="inlineStr">
+        <is>
+          <t>🟢 已就緒上線</t>
+        </is>
+      </c>
+      <c r="L27" t="inlineStr">
+        <is>
+          <t>A4 向量精編、一頁一題無縫排版、三色螢光筆印刷相容</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="n">
+        <v>24</v>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>第 2 課 觀點篇</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>應用文類講義</t>
+        </is>
+      </c>
+      <c r="D28" t="inlineStr">
+        <is>
+          <t>10_觀點篇_應用文類_詳解講義.pdf</t>
+        </is>
+      </c>
+      <c r="E28" t="inlineStr">
+        <is>
+          <t>10_viewpoint_practical_handout.pdf</t>
+        </is>
+      </c>
+      <c r="F28" t="inlineStr">
+        <is>
+          <t>P.40 ~ P.42</t>
+        </is>
+      </c>
+      <c r="G28" t="inlineStr">
+        <is>
+          <t>10 頁 (10題)</t>
+        </is>
+      </c>
+      <c r="H28" t="inlineStr">
+        <is>
+          <t>A4 單元精編詳解講義。含三色擬真螢光筆脈絡標註、解題之眼直擊死穴、白話語譯與逐項剖析。</t>
+        </is>
+      </c>
+      <c r="I28" t="inlineStr">
+        <is>
+          <t>https://oaoadna-1313.github.io/2026-literarymeaning8lesson/10_viewpoint_practical_handout.pdf</t>
+        </is>
+      </c>
+      <c r="J28" t="inlineStr">
+        <is>
+          <t>https://github.com/oaoadna-1313/2026-literarymeaning8lesson/blob/main/10_viewpoint_practical_handout.pdf</t>
+        </is>
+      </c>
+      <c r="K28" t="inlineStr">
+        <is>
+          <t>🟢 已就緒上線</t>
+        </is>
+      </c>
+      <c r="L28" t="inlineStr">
+        <is>
+          <t>A4 向量精編、一頁一題無縫排版、三色螢光筆印刷相容</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="n">
+        <v>25</v>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>第 2 課 觀點篇</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>全套合訂本講義</t>
+        </is>
+      </c>
+      <c r="D29" t="inlineStr">
+        <is>
+          <t>文意新8課_第2課觀點篇_全套精編詳解講義.pdf</t>
+        </is>
+      </c>
+      <c r="E29" t="inlineStr">
+        <is>
+          <t>02_viewpoint_complete_handout.pdf</t>
+        </is>
+      </c>
+      <c r="F29" t="inlineStr">
+        <is>
+          <t>P.28 ~ P.42</t>
+        </is>
+      </c>
+      <c r="G29" t="inlineStr">
+        <is>
+          <t>52 頁 (50題全解)</t>
+        </is>
+      </c>
+      <c r="H29" t="inlineStr">
+        <is>
+          <t>52 頁全套大合訂本。含典雅封面、單元目錄索引、會考解題策略心法、5 大文類 50 道實戰題完整精解。</t>
+        </is>
+      </c>
+      <c r="I29" t="inlineStr">
+        <is>
+          <t>https://oaoadna-1313.github.io/2026-literarymeaning8lesson/02_viewpoint_complete_handout.pdf</t>
+        </is>
+      </c>
+      <c r="J29" t="inlineStr">
+        <is>
+          <t>https://github.com/oaoadna-1313/2026-literarymeaning8lesson/blob/main/02_viewpoint_complete_handout.pdf</t>
+        </is>
+      </c>
+      <c r="K29" t="inlineStr">
+        <is>
+          <t>🟢 已就緒上線</t>
+        </is>
+      </c>
+      <c r="L29" t="inlineStr">
+        <is>
+          <t>典雅封面、單元目錄索引、使用指南與解題心法、50題一頁一題無縫精編</t>
         </is>
       </c>
     </row>
@@ -1747,7 +2407,7 @@
       </c>
       <c r="J10" s="25" t="inlineStr">
         <is>
-          <t>⚪ 準備中 (待產出)</t>
+          <t>🟢 已上線部署</t>
         </is>
       </c>
     </row>
@@ -1799,7 +2459,7 @@
       </c>
       <c r="J11" s="25" t="inlineStr">
         <is>
-          <t>⚪ 準備中 (待產出)</t>
+          <t>🟢 已上線部署</t>
         </is>
       </c>
     </row>
@@ -1851,7 +2511,7 @@
       </c>
       <c r="J12" s="25" t="inlineStr">
         <is>
-          <t>⚪ 準備中 (待產出)</t>
+          <t>🟢 已上線部署</t>
         </is>
       </c>
     </row>
@@ -1903,7 +2563,7 @@
       </c>
       <c r="J13" s="25" t="inlineStr">
         <is>
-          <t>⚪ 準備中 (待產出)</t>
+          <t>🟢 已上線部署</t>
         </is>
       </c>
     </row>
@@ -1955,7 +2615,7 @@
       </c>
       <c r="J14" s="25" t="inlineStr">
         <is>
-          <t>⚪ 準備中 (待產出)</t>
+          <t>🟢 已上線部署</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
feat: deploy Lesson 03 (Implication) interactive courseware, A4 handouts, complete collection PDF, and updated index
</commit_message>
<xml_diff>
--- a/文意新8課_GitHub部署檔案清單與網址對照表.xlsx
+++ b/文意新8課_GitHub部署檔案清單與網址對照表.xlsx
@@ -575,7 +575,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L29"/>
+  <dimension ref="A1:L40"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -606,7 +606,6 @@
         </is>
       </c>
     </row>
-    <row r="3"/>
     <row r="4" ht="28" customHeight="1">
       <c r="A4" s="3" t="inlineStr">
         <is>
@@ -1984,6 +1983,666 @@
         </is>
       </c>
       <c r="L29" t="inlineStr">
+        <is>
+          <t>典雅封面、單元目錄索引、使用指南與解題心法、50題一頁一題無縫精編</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="n">
+        <v>26</v>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>第 3 課 意涵篇</t>
+        </is>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>記敘文類</t>
+        </is>
+      </c>
+      <c r="D30" t="inlineStr">
+        <is>
+          <t>11_意涵篇_記敘文類.html</t>
+        </is>
+      </c>
+      <c r="E30" t="inlineStr">
+        <is>
+          <t>11_implication_narrative.html</t>
+        </is>
+      </c>
+      <c r="F30" t="inlineStr">
+        <is>
+          <t>P.48 ~ P.50</t>
+        </is>
+      </c>
+      <c r="G30" t="inlineStr">
+        <is>
+          <t>10 題</t>
+        </is>
+      </c>
+      <c r="H30" t="inlineStr">
+        <is>
+          <t>記敘文文句意涵與言外之意剖析。掌握作者在敘事敘景中寄託的深層意涵、弦外之音與象徵手法。</t>
+        </is>
+      </c>
+      <c r="I30" t="inlineStr">
+        <is>
+          <t>https://oaoadna-1313.github.io/2026-literarymeaning8lesson/11_implication_narrative.html</t>
+        </is>
+      </c>
+      <c r="J30" t="inlineStr">
+        <is>
+          <t>https://github.com/oaoadna-1313/2026-literarymeaning8lesson/blob/main/11_implication_narrative.html</t>
+        </is>
+      </c>
+      <c r="K30" t="inlineStr">
+        <is>
+          <t>🟢 已就緒上線</t>
+        </is>
+      </c>
+      <c r="L30" t="inlineStr">
+        <is>
+          <t>純題模式、即時答題回饋、多色螢光筆文本高亮、逐選項深度剖析、字級縮放</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="n">
+        <v>27</v>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>第 3 課 意涵篇</t>
+        </is>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>抒情文類</t>
+        </is>
+      </c>
+      <c r="D31" t="inlineStr">
+        <is>
+          <t>12_意涵篇_抒情文類.html</t>
+        </is>
+      </c>
+      <c r="E31" t="inlineStr">
+        <is>
+          <t>12_implication_lyric.html</t>
+        </is>
+      </c>
+      <c r="F31" t="inlineStr">
+        <is>
+          <t>P.51 ~ P.53</t>
+        </is>
+      </c>
+      <c r="G31" t="inlineStr">
+        <is>
+          <t>10 題</t>
+        </is>
+      </c>
+      <c r="H31" t="inlineStr">
+        <is>
+          <t>抒情文深層意涵與詩文意象解構。體察字句意蘊、藉物抒懷與情感層次轉換。</t>
+        </is>
+      </c>
+      <c r="I31" t="inlineStr">
+        <is>
+          <t>https://oaoadna-1313.github.io/2026-literarymeaning8lesson/12_implication_lyric.html</t>
+        </is>
+      </c>
+      <c r="J31" t="inlineStr">
+        <is>
+          <t>https://github.com/oaoadna-1313/2026-literarymeaning8lesson/blob/main/12_implication_lyric.html</t>
+        </is>
+      </c>
+      <c r="K31" t="inlineStr">
+        <is>
+          <t>🟢 已就緒上線</t>
+        </is>
+      </c>
+      <c r="L31" t="inlineStr">
+        <is>
+          <t>純題模式、即時答題回饋、情意核心高亮標註、完整語譯與注釋、錯題記錄</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="n">
+        <v>28</v>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>第 3 課 意涵篇</t>
+        </is>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>議論文類</t>
+        </is>
+      </c>
+      <c r="D32" t="inlineStr">
+        <is>
+          <t>13_意涵篇_議論文類.html</t>
+        </is>
+      </c>
+      <c r="E32" t="inlineStr">
+        <is>
+          <t>13_implication_argumentative.html</t>
+        </is>
+      </c>
+      <c r="F32" t="inlineStr">
+        <is>
+          <t>P.54 ~ P.56</t>
+        </is>
+      </c>
+      <c r="G32" t="inlineStr">
+        <is>
+          <t>10 題</t>
+        </is>
+      </c>
+      <c r="H32" t="inlineStr">
+        <is>
+          <t>議論文核心論述意涵與邏輯辨析。解碼論述文關鍵語句意涵、隱含假設與正反思辨脈絡。</t>
+        </is>
+      </c>
+      <c r="I32" t="inlineStr">
+        <is>
+          <t>https://oaoadna-1313.github.io/2026-literarymeaning8lesson/13_implication_argumentative.html</t>
+        </is>
+      </c>
+      <c r="J32" t="inlineStr">
+        <is>
+          <t>https://github.com/oaoadna-1313/2026-literarymeaning8lesson/blob/main/13_implication_argumentative.html</t>
+        </is>
+      </c>
+      <c r="K32" t="inlineStr">
+        <is>
+          <t>🟢 已就緒上線</t>
+        </is>
+      </c>
+      <c r="L32" t="inlineStr">
+        <is>
+          <t>解題之眼關鍵線索、論點句子動態螢光筆定位、逐項正誤解析、題號快速導覽</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="n">
+        <v>29</v>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>第 3 課 意涵篇</t>
+        </is>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>說明文類</t>
+        </is>
+      </c>
+      <c r="D33" t="inlineStr">
+        <is>
+          <t>14_意涵篇_說明文類.html</t>
+        </is>
+      </c>
+      <c r="E33" t="inlineStr">
+        <is>
+          <t>14_implication_expository.html</t>
+        </is>
+      </c>
+      <c r="F33" t="inlineStr">
+        <is>
+          <t>P.57 ~ P.59</t>
+        </is>
+      </c>
+      <c r="G33" t="inlineStr">
+        <is>
+          <t>10 題</t>
+        </is>
+      </c>
+      <c r="H33" t="inlineStr">
+        <is>
+          <t>說明文專業術語、文意表述與資訊內涵解讀。掌握科學、文化、生活說明文之精確意涵。</t>
+        </is>
+      </c>
+      <c r="I33" t="inlineStr">
+        <is>
+          <t>https://oaoadna-1313.github.io/2026-literarymeaning8lesson/14_implication_expository.html</t>
+        </is>
+      </c>
+      <c r="J33" t="inlineStr">
+        <is>
+          <t>https://github.com/oaoadna-1313/2026-literarymeaning8lesson/blob/main/14_implication_expository.html</t>
+        </is>
+      </c>
+      <c r="K33" t="inlineStr">
+        <is>
+          <t>🟢 已就緒上線</t>
+        </is>
+      </c>
+      <c r="L33" t="inlineStr">
+        <is>
+          <t>科技科普條理標註、文本知識架構拆解、互動單題/連續切換模式</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="n">
+        <v>30</v>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>第 3 課 意涵篇</t>
+        </is>
+      </c>
+      <c r="C34" t="inlineStr">
+        <is>
+          <t>應用文類</t>
+        </is>
+      </c>
+      <c r="D34" t="inlineStr">
+        <is>
+          <t>15_意涵篇_應用文類.html</t>
+        </is>
+      </c>
+      <c r="E34" t="inlineStr">
+        <is>
+          <t>15_implication_practical.html</t>
+        </is>
+      </c>
+      <c r="F34" t="inlineStr">
+        <is>
+          <t>P.60 ~ P.62</t>
+        </is>
+      </c>
+      <c r="G34" t="inlineStr">
+        <is>
+          <t>10 題</t>
+        </is>
+      </c>
+      <c r="H34" t="inlineStr">
+        <is>
+          <t>應用文語境意涵、特定格式表意與實用情境辨析。解讀書信、啟事、宣傳、聯對之用語意涵。</t>
+        </is>
+      </c>
+      <c r="I34" t="inlineStr">
+        <is>
+          <t>https://oaoadna-1313.github.io/2026-literarymeaning8lesson/15_implication_practical.html</t>
+        </is>
+      </c>
+      <c r="J34" t="inlineStr">
+        <is>
+          <t>https://github.com/oaoadna-1313/2026-literarymeaning8lesson/blob/main/15_implication_practical.html</t>
+        </is>
+      </c>
+      <c r="K34" t="inlineStr">
+        <is>
+          <t>🟢 已就緒上線</t>
+        </is>
+      </c>
+      <c r="L34" t="inlineStr">
+        <is>
+          <t>情境模擬文本、圖文閱讀重點對應高亮、生活素養題組深度解構</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="n">
+        <v>31</v>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>第 3 課 意涵篇</t>
+        </is>
+      </c>
+      <c r="C35" t="inlineStr">
+        <is>
+          <t>記敘文類講義</t>
+        </is>
+      </c>
+      <c r="D35" t="inlineStr">
+        <is>
+          <t>11_意涵篇_記敘文類_詳解講義.pdf</t>
+        </is>
+      </c>
+      <c r="E35" t="inlineStr">
+        <is>
+          <t>11_implication_narrative_handout.pdf</t>
+        </is>
+      </c>
+      <c r="F35" t="inlineStr">
+        <is>
+          <t>P.48 ~ P.50</t>
+        </is>
+      </c>
+      <c r="G35" t="inlineStr">
+        <is>
+          <t>10 頁 (10題)</t>
+        </is>
+      </c>
+      <c r="H35" t="inlineStr">
+        <is>
+          <t>A4 單元精編詳解講義。含三色擬真螢光筆脈絡標註、解題之眼直擊死穴、白話語譯與逐項剖析。</t>
+        </is>
+      </c>
+      <c r="I35" t="inlineStr">
+        <is>
+          <t>https://oaoadna-1313.github.io/2026-literarymeaning8lesson/11_implication_narrative_handout.pdf</t>
+        </is>
+      </c>
+      <c r="J35" t="inlineStr">
+        <is>
+          <t>https://github.com/oaoadna-1313/2026-literarymeaning8lesson/blob/main/11_implication_narrative_handout.pdf</t>
+        </is>
+      </c>
+      <c r="K35" t="inlineStr">
+        <is>
+          <t>🟢 已就緒上線</t>
+        </is>
+      </c>
+      <c r="L35" t="inlineStr">
+        <is>
+          <t>A4 向量精編、一頁一題無縫排版、三色螢光筆印刷相容</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="n">
+        <v>32</v>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>第 3 課 意涵篇</t>
+        </is>
+      </c>
+      <c r="C36" t="inlineStr">
+        <is>
+          <t>抒情文類講義</t>
+        </is>
+      </c>
+      <c r="D36" t="inlineStr">
+        <is>
+          <t>12_意涵篇_抒情文類_詳解講義.pdf</t>
+        </is>
+      </c>
+      <c r="E36" t="inlineStr">
+        <is>
+          <t>12_implication_lyric_handout.pdf</t>
+        </is>
+      </c>
+      <c r="F36" t="inlineStr">
+        <is>
+          <t>P.51 ~ P.53</t>
+        </is>
+      </c>
+      <c r="G36" t="inlineStr">
+        <is>
+          <t>10 頁 (10題)</t>
+        </is>
+      </c>
+      <c r="H36" t="inlineStr">
+        <is>
+          <t>A4 單元精編詳解講義。含三色擬真螢光筆脈絡標註、解題之眼直擊死穴、白話語譯與逐項剖析。</t>
+        </is>
+      </c>
+      <c r="I36" t="inlineStr">
+        <is>
+          <t>https://oaoadna-1313.github.io/2026-literarymeaning8lesson/12_implication_lyric_handout.pdf</t>
+        </is>
+      </c>
+      <c r="J36" t="inlineStr">
+        <is>
+          <t>https://github.com/oaoadna-1313/2026-literarymeaning8lesson/blob/main/12_implication_lyric_handout.pdf</t>
+        </is>
+      </c>
+      <c r="K36" t="inlineStr">
+        <is>
+          <t>🟢 已就緒上線</t>
+        </is>
+      </c>
+      <c r="L36" t="inlineStr">
+        <is>
+          <t>A4 向量精編、一頁一題無縫排版、三色螢光筆印刷相容</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="n">
+        <v>33</v>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>第 3 課 意涵篇</t>
+        </is>
+      </c>
+      <c r="C37" t="inlineStr">
+        <is>
+          <t>議論文類講義</t>
+        </is>
+      </c>
+      <c r="D37" t="inlineStr">
+        <is>
+          <t>13_意涵篇_議論文類_詳解講義.pdf</t>
+        </is>
+      </c>
+      <c r="E37" t="inlineStr">
+        <is>
+          <t>13_implication_argumentative_handout.pdf</t>
+        </is>
+      </c>
+      <c r="F37" t="inlineStr">
+        <is>
+          <t>P.54 ~ P.56</t>
+        </is>
+      </c>
+      <c r="G37" t="inlineStr">
+        <is>
+          <t>10 頁 (10題)</t>
+        </is>
+      </c>
+      <c r="H37" t="inlineStr">
+        <is>
+          <t>A4 單元精編詳解講義。含三色擬真螢光筆脈絡標註、解題之眼直擊死穴、白話語譯與逐項剖析。</t>
+        </is>
+      </c>
+      <c r="I37" t="inlineStr">
+        <is>
+          <t>https://oaoadna-1313.github.io/2026-literarymeaning8lesson/13_implication_argumentative_handout.pdf</t>
+        </is>
+      </c>
+      <c r="J37" t="inlineStr">
+        <is>
+          <t>https://github.com/oaoadna-1313/2026-literarymeaning8lesson/blob/main/13_implication_argumentative_handout.pdf</t>
+        </is>
+      </c>
+      <c r="K37" t="inlineStr">
+        <is>
+          <t>🟢 已就緒上線</t>
+        </is>
+      </c>
+      <c r="L37" t="inlineStr">
+        <is>
+          <t>A4 向量精編、一頁一題無縫排版、三色螢光筆印刷相容</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="n">
+        <v>34</v>
+      </c>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>第 3 課 意涵篇</t>
+        </is>
+      </c>
+      <c r="C38" t="inlineStr">
+        <is>
+          <t>說明文類講義</t>
+        </is>
+      </c>
+      <c r="D38" t="inlineStr">
+        <is>
+          <t>14_意涵篇_說明文類_詳解講義.pdf</t>
+        </is>
+      </c>
+      <c r="E38" t="inlineStr">
+        <is>
+          <t>14_implication_expository_handout.pdf</t>
+        </is>
+      </c>
+      <c r="F38" t="inlineStr">
+        <is>
+          <t>P.57 ~ P.59</t>
+        </is>
+      </c>
+      <c r="G38" t="inlineStr">
+        <is>
+          <t>10 頁 (10題)</t>
+        </is>
+      </c>
+      <c r="H38" t="inlineStr">
+        <is>
+          <t>A4 單元精編詳解講義。含三色擬真螢光筆脈絡標註、解題之眼直擊死穴、白話語譯與逐項剖析。</t>
+        </is>
+      </c>
+      <c r="I38" t="inlineStr">
+        <is>
+          <t>https://oaoadna-1313.github.io/2026-literarymeaning8lesson/14_implication_expository_handout.pdf</t>
+        </is>
+      </c>
+      <c r="J38" t="inlineStr">
+        <is>
+          <t>https://github.com/oaoadna-1313/2026-literarymeaning8lesson/blob/main/14_implication_expository_handout.pdf</t>
+        </is>
+      </c>
+      <c r="K38" t="inlineStr">
+        <is>
+          <t>🟢 已就緒上線</t>
+        </is>
+      </c>
+      <c r="L38" t="inlineStr">
+        <is>
+          <t>A4 向量精編、一頁一題無縫排版、三色螢光筆印刷相容</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="n">
+        <v>35</v>
+      </c>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>第 3 課 意涵篇</t>
+        </is>
+      </c>
+      <c r="C39" t="inlineStr">
+        <is>
+          <t>應用文類講義</t>
+        </is>
+      </c>
+      <c r="D39" t="inlineStr">
+        <is>
+          <t>15_意涵篇_應用文類_詳解講義.pdf</t>
+        </is>
+      </c>
+      <c r="E39" t="inlineStr">
+        <is>
+          <t>15_implication_practical_handout.pdf</t>
+        </is>
+      </c>
+      <c r="F39" t="inlineStr">
+        <is>
+          <t>P.60 ~ P.62</t>
+        </is>
+      </c>
+      <c r="G39" t="inlineStr">
+        <is>
+          <t>10 頁 (10題)</t>
+        </is>
+      </c>
+      <c r="H39" t="inlineStr">
+        <is>
+          <t>A4 單元精編詳解講義。含三色擬真螢光筆脈絡標註、解題之眼直擊死穴、白話語譯與逐項剖析。</t>
+        </is>
+      </c>
+      <c r="I39" t="inlineStr">
+        <is>
+          <t>https://oaoadna-1313.github.io/2026-literarymeaning8lesson/15_implication_practical_handout.pdf</t>
+        </is>
+      </c>
+      <c r="J39" t="inlineStr">
+        <is>
+          <t>https://github.com/oaoadna-1313/2026-literarymeaning8lesson/blob/main/15_implication_practical_handout.pdf</t>
+        </is>
+      </c>
+      <c r="K39" t="inlineStr">
+        <is>
+          <t>🟢 已就緒上線</t>
+        </is>
+      </c>
+      <c r="L39" t="inlineStr">
+        <is>
+          <t>A4 向量精編、一頁一題無縫排版、三色螢光筆印刷相容</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="n">
+        <v>36</v>
+      </c>
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>第 3 課 意涵篇</t>
+        </is>
+      </c>
+      <c r="C40" t="inlineStr">
+        <is>
+          <t>全套合訂本講義</t>
+        </is>
+      </c>
+      <c r="D40" t="inlineStr">
+        <is>
+          <t>文意新8課_第3課意涵篇_全套精編詳解講義.pdf</t>
+        </is>
+      </c>
+      <c r="E40" t="inlineStr">
+        <is>
+          <t>03_implication_complete_handout.pdf</t>
+        </is>
+      </c>
+      <c r="F40" t="inlineStr">
+        <is>
+          <t>P.48 ~ P.62</t>
+        </is>
+      </c>
+      <c r="G40" t="inlineStr">
+        <is>
+          <t>52 頁 (50題全解)</t>
+        </is>
+      </c>
+      <c r="H40" t="inlineStr">
+        <is>
+          <t>52 頁全套大合訂本。含典雅封面、單元目錄索引、會考解題策略心法、5 大文類 50 道實戰題完整精解。</t>
+        </is>
+      </c>
+      <c r="I40" t="inlineStr">
+        <is>
+          <t>https://oaoadna-1313.github.io/2026-literarymeaning8lesson/03_implication_complete_handout.pdf</t>
+        </is>
+      </c>
+      <c r="J40" t="inlineStr">
+        <is>
+          <t>https://github.com/oaoadna-1313/2026-literarymeaning8lesson/blob/main/03_implication_complete_handout.pdf</t>
+        </is>
+      </c>
+      <c r="K40" t="inlineStr">
+        <is>
+          <t>🟢 已就緒上線</t>
+        </is>
+      </c>
+      <c r="L40" t="inlineStr">
         <is>
           <t>典雅封面、單元目錄索引、使用指南與解題心法、50題一頁一題無縫精編</t>
         </is>
@@ -2667,7 +3326,7 @@
       </c>
       <c r="J15" s="25" t="inlineStr">
         <is>
-          <t>⚪ 準備中 (待產出)</t>
+          <t>🟢 已上線部署</t>
         </is>
       </c>
     </row>
@@ -2719,7 +3378,7 @@
       </c>
       <c r="J16" s="25" t="inlineStr">
         <is>
-          <t>⚪ 準備中 (待產出)</t>
+          <t>🟢 已上線部署</t>
         </is>
       </c>
     </row>
@@ -2771,7 +3430,7 @@
       </c>
       <c r="J17" s="25" t="inlineStr">
         <is>
-          <t>⚪ 準備中 (待產出)</t>
+          <t>🟢 已上線部署</t>
         </is>
       </c>
     </row>
@@ -2823,7 +3482,7 @@
       </c>
       <c r="J18" s="25" t="inlineStr">
         <is>
-          <t>⚪ 準備中 (待產出)</t>
+          <t>🟢 已上線部署</t>
         </is>
       </c>
     </row>
@@ -2875,7 +3534,7 @@
       </c>
       <c r="J19" s="25" t="inlineStr">
         <is>
-          <t>⚪ 準備中 (待產出)</t>
+          <t>🟢 已上線部署</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
feat: add Unit 38 and 39 review assessments (1 & 2) interactive courseware, handouts and complete collection PDF
</commit_message>
<xml_diff>
--- a/文意新8課_GitHub部署檔案清單與網址對照表.xlsx
+++ b/文意新8課_GitHub部署檔案清單與網址對照表.xlsx
@@ -18,7 +18,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="9">
+  <fonts count="12">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -72,8 +72,23 @@
       <color rgb="0094A3B8"/>
       <sz val="10"/>
     </font>
+    <font>
+      <name val="Microsoft JhengHei"/>
+      <sz val="9.5"/>
+    </font>
+    <font>
+      <name val="Microsoft JhengHei"/>
+      <color rgb="000284C7"/>
+      <sz val="9.5"/>
+      <u val="single"/>
+    </font>
+    <font>
+      <name val="Microsoft JhengHei"/>
+      <b val="1"/>
+      <sz val="9.5"/>
+    </font>
   </fonts>
-  <fills count="7">
+  <fills count="8">
     <fill>
       <patternFill/>
     </fill>
@@ -110,6 +125,12 @@
         <bgColor rgb="000F766E"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FFFFFF"/>
+        <bgColor rgb="00FFFFFF"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="2">
     <border>
@@ -137,7 +158,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="26">
+  <cellXfs count="33">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -209,6 +230,27 @@
     </xf>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -575,7 +617,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L40"/>
+  <dimension ref="A1:L94"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -606,6 +648,7 @@
         </is>
       </c>
     </row>
+    <row r="3"/>
     <row r="4" ht="28" customHeight="1">
       <c r="A4" s="3" t="inlineStr">
         <is>
@@ -2645,6 +2688,3246 @@
       <c r="L40" t="inlineStr">
         <is>
           <t>典雅封面、單元目錄索引、使用指南與解題心法、50題一頁一題無縫精編</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="26" t="n">
+        <v>37</v>
+      </c>
+      <c r="B41" s="27" t="inlineStr">
+        <is>
+          <t>第 4 課 解釋篇</t>
+        </is>
+      </c>
+      <c r="C41" s="27" t="inlineStr">
+        <is>
+          <t>記敘文類</t>
+        </is>
+      </c>
+      <c r="D41" s="27" t="inlineStr">
+        <is>
+          <t>16_解釋篇_記敘文類.html</t>
+        </is>
+      </c>
+      <c r="E41" s="27" t="inlineStr">
+        <is>
+          <t>16_interpretation_narrative.html</t>
+        </is>
+      </c>
+      <c r="F41" s="26" t="inlineStr">
+        <is>
+          <t>P.68 ~ P.70</t>
+        </is>
+      </c>
+      <c r="G41" s="26" t="inlineStr">
+        <is>
+          <t>10 題</t>
+        </is>
+      </c>
+      <c r="H41" s="27" t="inlineStr">
+        <is>
+          <t>記敘文詞意代入與文境轉換</t>
+        </is>
+      </c>
+      <c r="I41" s="28" t="inlineStr">
+        <is>
+          <t>https://oaoadna-1313.github.io/2026-literarymeaning8lesson/16_interpretation_narrative.html</t>
+        </is>
+      </c>
+      <c r="J41" s="28" t="inlineStr">
+        <is>
+          <t>https://github.com/oaoadna-1313/2026-literarymeaning8lesson/blob/main/16_interpretation_narrative.html</t>
+        </is>
+      </c>
+      <c r="K41" s="29" t="inlineStr">
+        <is>
+          <t>✅ 100% 完成上線</t>
+        </is>
+      </c>
+      <c r="L41" s="27" t="inlineStr">
+        <is>
+          <t>雙軌切換・三色螢光筆・解題之眼・逐項剖析</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="30" t="n">
+        <v>38</v>
+      </c>
+      <c r="B42" s="31" t="inlineStr">
+        <is>
+          <t>第 4 課 解釋篇</t>
+        </is>
+      </c>
+      <c r="C42" s="31" t="inlineStr">
+        <is>
+          <t>抒情文類</t>
+        </is>
+      </c>
+      <c r="D42" s="31" t="inlineStr">
+        <is>
+          <t>17_解釋篇_抒情文類.html</t>
+        </is>
+      </c>
+      <c r="E42" s="31" t="inlineStr">
+        <is>
+          <t>17_interpretation_lyric.html</t>
+        </is>
+      </c>
+      <c r="F42" s="30" t="inlineStr">
+        <is>
+          <t>P.71 ~ P.73</t>
+        </is>
+      </c>
+      <c r="G42" s="30" t="inlineStr">
+        <is>
+          <t>8 題</t>
+        </is>
+      </c>
+      <c r="H42" s="31" t="inlineStr">
+        <is>
+          <t>抒情文情境意象轉化與情感詮釋</t>
+        </is>
+      </c>
+      <c r="I42" s="32" t="inlineStr">
+        <is>
+          <t>https://oaoadna-1313.github.io/2026-literarymeaning8lesson/17_interpretation_lyric.html</t>
+        </is>
+      </c>
+      <c r="J42" s="32" t="inlineStr">
+        <is>
+          <t>https://github.com/oaoadna-1313/2026-literarymeaning8lesson/blob/main/17_interpretation_lyric.html</t>
+        </is>
+      </c>
+      <c r="K42" s="29" t="inlineStr">
+        <is>
+          <t>✅ 100% 完成上線</t>
+        </is>
+      </c>
+      <c r="L42" s="31" t="inlineStr">
+        <is>
+          <t>雙軌切換・三色螢光筆・解題之眼・逐項剖析</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="26" t="n">
+        <v>39</v>
+      </c>
+      <c r="B43" s="27" t="inlineStr">
+        <is>
+          <t>第 4 課 解釋篇</t>
+        </is>
+      </c>
+      <c r="C43" s="27" t="inlineStr">
+        <is>
+          <t>議論文類</t>
+        </is>
+      </c>
+      <c r="D43" s="27" t="inlineStr">
+        <is>
+          <t>18_解釋篇_議論文類.html</t>
+        </is>
+      </c>
+      <c r="E43" s="27" t="inlineStr">
+        <is>
+          <t>18_interpretation_argumentative.html</t>
+        </is>
+      </c>
+      <c r="F43" s="26" t="inlineStr">
+        <is>
+          <t>P.74 ~ P.76</t>
+        </is>
+      </c>
+      <c r="G43" s="26" t="inlineStr">
+        <is>
+          <t>8 題</t>
+        </is>
+      </c>
+      <c r="H43" s="27" t="inlineStr">
+        <is>
+          <t>議論文名詞界定、論點釐清與論據反詰</t>
+        </is>
+      </c>
+      <c r="I43" s="28" t="inlineStr">
+        <is>
+          <t>https://oaoadna-1313.github.io/2026-literarymeaning8lesson/18_interpretation_argumentative.html</t>
+        </is>
+      </c>
+      <c r="J43" s="28" t="inlineStr">
+        <is>
+          <t>https://github.com/oaoadna-1313/2026-literarymeaning8lesson/blob/main/18_interpretation_argumentative.html</t>
+        </is>
+      </c>
+      <c r="K43" s="29" t="inlineStr">
+        <is>
+          <t>✅ 100% 完成上線</t>
+        </is>
+      </c>
+      <c r="L43" s="27" t="inlineStr">
+        <is>
+          <t>雙軌切換・三色螢光筆・解題之眼・逐項剖析</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="30" t="n">
+        <v>40</v>
+      </c>
+      <c r="B44" s="31" t="inlineStr">
+        <is>
+          <t>第 4 課 解釋篇</t>
+        </is>
+      </c>
+      <c r="C44" s="31" t="inlineStr">
+        <is>
+          <t>說明文類</t>
+        </is>
+      </c>
+      <c r="D44" s="31" t="inlineStr">
+        <is>
+          <t>19_解釋篇_說明文類.html</t>
+        </is>
+      </c>
+      <c r="E44" s="31" t="inlineStr">
+        <is>
+          <t>19_interpretation_expository.html</t>
+        </is>
+      </c>
+      <c r="F44" s="30" t="inlineStr">
+        <is>
+          <t>P.77 ~ P.79</t>
+        </is>
+      </c>
+      <c r="G44" s="30" t="inlineStr">
+        <is>
+          <t>6 題</t>
+        </is>
+      </c>
+      <c r="H44" s="31" t="inlineStr">
+        <is>
+          <t>說明文科學概念詮釋與定義置換</t>
+        </is>
+      </c>
+      <c r="I44" s="32" t="inlineStr">
+        <is>
+          <t>https://oaoadna-1313.github.io/2026-literarymeaning8lesson/19_interpretation_expository.html</t>
+        </is>
+      </c>
+      <c r="J44" s="32" t="inlineStr">
+        <is>
+          <t>https://github.com/oaoadna-1313/2026-literarymeaning8lesson/blob/main/19_interpretation_expository.html</t>
+        </is>
+      </c>
+      <c r="K44" s="29" t="inlineStr">
+        <is>
+          <t>✅ 100% 完成上線</t>
+        </is>
+      </c>
+      <c r="L44" s="31" t="inlineStr">
+        <is>
+          <t>雙軌切換・三色螢光筆・解題之眼・逐項剖析</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="26" t="n">
+        <v>41</v>
+      </c>
+      <c r="B45" s="27" t="inlineStr">
+        <is>
+          <t>第 4 課 解釋篇</t>
+        </is>
+      </c>
+      <c r="C45" s="27" t="inlineStr">
+        <is>
+          <t>應用文類</t>
+        </is>
+      </c>
+      <c r="D45" s="27" t="inlineStr">
+        <is>
+          <t>20_解釋篇_應用文類.html</t>
+        </is>
+      </c>
+      <c r="E45" s="27" t="inlineStr">
+        <is>
+          <t>20_interpretation_practical.html</t>
+        </is>
+      </c>
+      <c r="F45" s="26" t="inlineStr">
+        <is>
+          <t>P.80 ~ P.82</t>
+        </is>
+      </c>
+      <c r="G45" s="26" t="inlineStr">
+        <is>
+          <t>9 題</t>
+        </is>
+      </c>
+      <c r="H45" s="27" t="inlineStr">
+        <is>
+          <t>應用文書信稱謂、題辭語意與生活規章</t>
+        </is>
+      </c>
+      <c r="I45" s="28" t="inlineStr">
+        <is>
+          <t>https://oaoadna-1313.github.io/2026-literarymeaning8lesson/20_interpretation_practical.html</t>
+        </is>
+      </c>
+      <c r="J45" s="28" t="inlineStr">
+        <is>
+          <t>https://github.com/oaoadna-1313/2026-literarymeaning8lesson/blob/main/20_interpretation_practical.html</t>
+        </is>
+      </c>
+      <c r="K45" s="29" t="inlineStr">
+        <is>
+          <t>✅ 100% 完成上線</t>
+        </is>
+      </c>
+      <c r="L45" s="27" t="inlineStr">
+        <is>
+          <t>雙軌切換・三色螢光筆・解題之眼・逐項剖析</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="30" t="n">
+        <v>42</v>
+      </c>
+      <c r="B46" s="31" t="inlineStr">
+        <is>
+          <t>第 4 課 解釋篇</t>
+        </is>
+      </c>
+      <c r="C46" s="31" t="inlineStr">
+        <is>
+          <t>記敘文類講義</t>
+        </is>
+      </c>
+      <c r="D46" s="31" t="inlineStr">
+        <is>
+          <t>16_解釋篇_記敘文類_詳解講義.pdf</t>
+        </is>
+      </c>
+      <c r="E46" s="31" t="inlineStr">
+        <is>
+          <t>16_interpretation_narrative_handout.pdf</t>
+        </is>
+      </c>
+      <c r="F46" s="30" t="inlineStr">
+        <is>
+          <t>P.68 ~ P.70</t>
+        </is>
+      </c>
+      <c r="G46" s="30" t="inlineStr">
+        <is>
+          <t>10 頁</t>
+        </is>
+      </c>
+      <c r="H46" s="31" t="inlineStr">
+        <is>
+          <t>A4單頁精編・三色螢光筆・解題之眼・語譯</t>
+        </is>
+      </c>
+      <c r="I46" s="32" t="inlineStr">
+        <is>
+          <t>https://oaoadna-1313.github.io/2026-literarymeaning8lesson/16_interpretation_narrative_handout.pdf</t>
+        </is>
+      </c>
+      <c r="J46" s="32" t="inlineStr">
+        <is>
+          <t>https://github.com/oaoadna-1313/2026-literarymeaning8lesson/blob/main/16_interpretation_narrative_handout.pdf</t>
+        </is>
+      </c>
+      <c r="K46" s="29" t="inlineStr">
+        <is>
+          <t>✅ 100% 完成上線</t>
+        </is>
+      </c>
+      <c r="L46" s="31" t="inlineStr">
+        <is>
+          <t>A4向量排版・一題一頁絕不溢出・精編詳解講義</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="26" t="n">
+        <v>43</v>
+      </c>
+      <c r="B47" s="27" t="inlineStr">
+        <is>
+          <t>第 4 課 解釋篇</t>
+        </is>
+      </c>
+      <c r="C47" s="27" t="inlineStr">
+        <is>
+          <t>抒情文類講義</t>
+        </is>
+      </c>
+      <c r="D47" s="27" t="inlineStr">
+        <is>
+          <t>17_解釋篇_抒情文類_詳解講義.pdf</t>
+        </is>
+      </c>
+      <c r="E47" s="27" t="inlineStr">
+        <is>
+          <t>17_interpretation_lyric_handout.pdf</t>
+        </is>
+      </c>
+      <c r="F47" s="26" t="inlineStr">
+        <is>
+          <t>P.71 ~ P.73</t>
+        </is>
+      </c>
+      <c r="G47" s="26" t="inlineStr">
+        <is>
+          <t>8 頁</t>
+        </is>
+      </c>
+      <c r="H47" s="27" t="inlineStr">
+        <is>
+          <t>A4單頁精編・三色螢光筆・解題之眼・語譯</t>
+        </is>
+      </c>
+      <c r="I47" s="28" t="inlineStr">
+        <is>
+          <t>https://oaoadna-1313.github.io/2026-literarymeaning8lesson/17_interpretation_lyric_handout.pdf</t>
+        </is>
+      </c>
+      <c r="J47" s="28" t="inlineStr">
+        <is>
+          <t>https://github.com/oaoadna-1313/2026-literarymeaning8lesson/blob/main/17_interpretation_lyric_handout.pdf</t>
+        </is>
+      </c>
+      <c r="K47" s="29" t="inlineStr">
+        <is>
+          <t>✅ 100% 完成上線</t>
+        </is>
+      </c>
+      <c r="L47" s="27" t="inlineStr">
+        <is>
+          <t>A4向量排版・一題一頁絕不溢出・精編詳解講義</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="30" t="n">
+        <v>44</v>
+      </c>
+      <c r="B48" s="31" t="inlineStr">
+        <is>
+          <t>第 4 課 解釋篇</t>
+        </is>
+      </c>
+      <c r="C48" s="31" t="inlineStr">
+        <is>
+          <t>議論文類講義</t>
+        </is>
+      </c>
+      <c r="D48" s="31" t="inlineStr">
+        <is>
+          <t>18_解釋篇_議論文類_詳解講義.pdf</t>
+        </is>
+      </c>
+      <c r="E48" s="31" t="inlineStr">
+        <is>
+          <t>18_interpretation_argumentative_handout.pdf</t>
+        </is>
+      </c>
+      <c r="F48" s="30" t="inlineStr">
+        <is>
+          <t>P.74 ~ P.76</t>
+        </is>
+      </c>
+      <c r="G48" s="30" t="inlineStr">
+        <is>
+          <t>8 頁</t>
+        </is>
+      </c>
+      <c r="H48" s="31" t="inlineStr">
+        <is>
+          <t>A4單頁精編・三色螢光筆・解題之眼・語譯</t>
+        </is>
+      </c>
+      <c r="I48" s="32" t="inlineStr">
+        <is>
+          <t>https://oaoadna-1313.github.io/2026-literarymeaning8lesson/18_interpretation_argumentative_handout.pdf</t>
+        </is>
+      </c>
+      <c r="J48" s="32" t="inlineStr">
+        <is>
+          <t>https://github.com/oaoadna-1313/2026-literarymeaning8lesson/blob/main/18_interpretation_argumentative_handout.pdf</t>
+        </is>
+      </c>
+      <c r="K48" s="29" t="inlineStr">
+        <is>
+          <t>✅ 100% 完成上線</t>
+        </is>
+      </c>
+      <c r="L48" s="31" t="inlineStr">
+        <is>
+          <t>A4向量排版・一題一頁絕不溢出・精編詳解講義</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="26" t="n">
+        <v>45</v>
+      </c>
+      <c r="B49" s="27" t="inlineStr">
+        <is>
+          <t>第 4 課 解釋篇</t>
+        </is>
+      </c>
+      <c r="C49" s="27" t="inlineStr">
+        <is>
+          <t>說明文類講義</t>
+        </is>
+      </c>
+      <c r="D49" s="27" t="inlineStr">
+        <is>
+          <t>19_解釋篇_說明文類_詳解講義.pdf</t>
+        </is>
+      </c>
+      <c r="E49" s="27" t="inlineStr">
+        <is>
+          <t>19_interpretation_expository_handout.pdf</t>
+        </is>
+      </c>
+      <c r="F49" s="26" t="inlineStr">
+        <is>
+          <t>P.77 ~ P.79</t>
+        </is>
+      </c>
+      <c r="G49" s="26" t="inlineStr">
+        <is>
+          <t>6 頁</t>
+        </is>
+      </c>
+      <c r="H49" s="27" t="inlineStr">
+        <is>
+          <t>A4單頁精編・三色螢光筆・解題之眼・語譯</t>
+        </is>
+      </c>
+      <c r="I49" s="28" t="inlineStr">
+        <is>
+          <t>https://oaoadna-1313.github.io/2026-literarymeaning8lesson/19_interpretation_expository_handout.pdf</t>
+        </is>
+      </c>
+      <c r="J49" s="28" t="inlineStr">
+        <is>
+          <t>https://github.com/oaoadna-1313/2026-literarymeaning8lesson/blob/main/19_interpretation_expository_handout.pdf</t>
+        </is>
+      </c>
+      <c r="K49" s="29" t="inlineStr">
+        <is>
+          <t>✅ 100% 完成上線</t>
+        </is>
+      </c>
+      <c r="L49" s="27" t="inlineStr">
+        <is>
+          <t>A4向量排版・一題一頁絕不溢出・精編詳解講義</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="30" t="n">
+        <v>46</v>
+      </c>
+      <c r="B50" s="31" t="inlineStr">
+        <is>
+          <t>第 4 課 解釋篇</t>
+        </is>
+      </c>
+      <c r="C50" s="31" t="inlineStr">
+        <is>
+          <t>應用文類講義</t>
+        </is>
+      </c>
+      <c r="D50" s="31" t="inlineStr">
+        <is>
+          <t>20_解釋篇_應用文類_詳解講義.pdf</t>
+        </is>
+      </c>
+      <c r="E50" s="31" t="inlineStr">
+        <is>
+          <t>20_interpretation_practical_handout.pdf</t>
+        </is>
+      </c>
+      <c r="F50" s="30" t="inlineStr">
+        <is>
+          <t>P.80 ~ P.82</t>
+        </is>
+      </c>
+      <c r="G50" s="30" t="inlineStr">
+        <is>
+          <t>9 頁</t>
+        </is>
+      </c>
+      <c r="H50" s="31" t="inlineStr">
+        <is>
+          <t>A4單頁精編・三色螢光筆・解題之眼・語譯</t>
+        </is>
+      </c>
+      <c r="I50" s="32" t="inlineStr">
+        <is>
+          <t>https://oaoadna-1313.github.io/2026-literarymeaning8lesson/20_interpretation_practical_handout.pdf</t>
+        </is>
+      </c>
+      <c r="J50" s="32" t="inlineStr">
+        <is>
+          <t>https://github.com/oaoadna-1313/2026-literarymeaning8lesson/blob/main/20_interpretation_practical_handout.pdf</t>
+        </is>
+      </c>
+      <c r="K50" s="29" t="inlineStr">
+        <is>
+          <t>✅ 100% 完成上線</t>
+        </is>
+      </c>
+      <c r="L50" s="31" t="inlineStr">
+        <is>
+          <t>A4向量排版・一題一頁絕不溢出・精編詳解講義</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="26" t="n">
+        <v>47</v>
+      </c>
+      <c r="B51" s="27" t="inlineStr">
+        <is>
+          <t>第 4 課 解釋篇</t>
+        </is>
+      </c>
+      <c r="C51" s="27" t="inlineStr">
+        <is>
+          <t>全套合訂本講義</t>
+        </is>
+      </c>
+      <c r="D51" s="27" t="inlineStr">
+        <is>
+          <t>文意新8課_第4課解釋篇_全套精編詳解講義.pdf</t>
+        </is>
+      </c>
+      <c r="E51" s="27" t="inlineStr">
+        <is>
+          <t>04_interpretation_complete_handout.pdf</t>
+        </is>
+      </c>
+      <c r="F51" s="26" t="inlineStr">
+        <is>
+          <t>全書 P.68~82</t>
+        </is>
+      </c>
+      <c r="G51" s="26" t="inlineStr">
+        <is>
+          <t>43 頁</t>
+        </is>
+      </c>
+      <c r="H51" s="27" t="inlineStr">
+        <is>
+          <t>全冊大合訂本：封面+總目錄+41題單頁精編</t>
+        </is>
+      </c>
+      <c r="I51" s="28" t="inlineStr">
+        <is>
+          <t>https://oaoadna-1313.github.io/2026-literarymeaning8lesson/04_interpretation_complete_handout.pdf</t>
+        </is>
+      </c>
+      <c r="J51" s="28" t="inlineStr">
+        <is>
+          <t>https://github.com/oaoadna-1313/2026-literarymeaning8lesson/blob/main/04_interpretation_complete_handout.pdf</t>
+        </is>
+      </c>
+      <c r="K51" s="29" t="inlineStr">
+        <is>
+          <t>✅ 100% 完成上線</t>
+        </is>
+      </c>
+      <c r="L51" s="27" t="inlineStr">
+        <is>
+          <t>A4向量排版・一題一頁絕不溢出・精編詳解講義</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" s="30" t="n">
+        <v>48</v>
+      </c>
+      <c r="B52" s="31" t="inlineStr">
+        <is>
+          <t>第 5 課 比較篇</t>
+        </is>
+      </c>
+      <c r="C52" s="31" t="inlineStr">
+        <is>
+          <t>記敘文類</t>
+        </is>
+      </c>
+      <c r="D52" s="31" t="inlineStr">
+        <is>
+          <t>21_比較篇_記敘文類.html</t>
+        </is>
+      </c>
+      <c r="E52" s="31" t="inlineStr">
+        <is>
+          <t>21_comparison_narrative.html</t>
+        </is>
+      </c>
+      <c r="F52" s="30" t="inlineStr">
+        <is>
+          <t>P.88 ~ P.91</t>
+        </is>
+      </c>
+      <c r="G52" s="30" t="inlineStr">
+        <is>
+          <t>8 題</t>
+        </is>
+      </c>
+      <c r="H52" s="31" t="inlineStr">
+        <is>
+          <t>雙篇記敘人物性格、事件觀點與行文手法比較</t>
+        </is>
+      </c>
+      <c r="I52" s="32" t="inlineStr">
+        <is>
+          <t>https://oaoadna-1313.github.io/2026-literarymeaning8lesson/21_comparison_narrative.html</t>
+        </is>
+      </c>
+      <c r="J52" s="32" t="inlineStr">
+        <is>
+          <t>https://github.com/oaoadna-1313/2026-literarymeaning8lesson/blob/main/21_comparison_narrative.html</t>
+        </is>
+      </c>
+      <c r="K52" s="29" t="inlineStr">
+        <is>
+          <t>✅ 100% 完成上線</t>
+        </is>
+      </c>
+      <c r="L52" s="31" t="inlineStr">
+        <is>
+          <t>雙軌切換・三色螢光筆・解題之眼・逐項剖析</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" s="26" t="n">
+        <v>49</v>
+      </c>
+      <c r="B53" s="27" t="inlineStr">
+        <is>
+          <t>第 5 課 比較篇</t>
+        </is>
+      </c>
+      <c r="C53" s="27" t="inlineStr">
+        <is>
+          <t>抒情文類</t>
+        </is>
+      </c>
+      <c r="D53" s="27" t="inlineStr">
+        <is>
+          <t>22_比較篇_抒情文類.html</t>
+        </is>
+      </c>
+      <c r="E53" s="27" t="inlineStr">
+        <is>
+          <t>22_comparison_lyric.html</t>
+        </is>
+      </c>
+      <c r="F53" s="26" t="inlineStr">
+        <is>
+          <t>P.92 ~ P.94</t>
+        </is>
+      </c>
+      <c r="G53" s="26" t="inlineStr">
+        <is>
+          <t>10 題</t>
+        </is>
+      </c>
+      <c r="H53" s="27" t="inlineStr">
+        <is>
+          <t>跨時代詩歌意境、情感寄託與生命情懷異同對比</t>
+        </is>
+      </c>
+      <c r="I53" s="28" t="inlineStr">
+        <is>
+          <t>https://oaoadna-1313.github.io/2026-literarymeaning8lesson/22_comparison_lyric.html</t>
+        </is>
+      </c>
+      <c r="J53" s="28" t="inlineStr">
+        <is>
+          <t>https://github.com/oaoadna-1313/2026-literarymeaning8lesson/blob/main/22_comparison_lyric.html</t>
+        </is>
+      </c>
+      <c r="K53" s="29" t="inlineStr">
+        <is>
+          <t>✅ 100% 完成上線</t>
+        </is>
+      </c>
+      <c r="L53" s="27" t="inlineStr">
+        <is>
+          <t>雙軌切換・三色螢光筆・解題之眼・逐項剖析</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" s="30" t="n">
+        <v>50</v>
+      </c>
+      <c r="B54" s="31" t="inlineStr">
+        <is>
+          <t>第 5 課 比較篇</t>
+        </is>
+      </c>
+      <c r="C54" s="31" t="inlineStr">
+        <is>
+          <t>議論文類</t>
+        </is>
+      </c>
+      <c r="D54" s="31" t="inlineStr">
+        <is>
+          <t>23_比較篇_議論文類.html</t>
+        </is>
+      </c>
+      <c r="E54" s="31" t="inlineStr">
+        <is>
+          <t>23_comparison_argumentative.html</t>
+        </is>
+      </c>
+      <c r="F54" s="30" t="inlineStr">
+        <is>
+          <t>P.95 ~ P.97</t>
+        </is>
+      </c>
+      <c r="G54" s="30" t="inlineStr">
+        <is>
+          <t>10 題</t>
+        </is>
+      </c>
+      <c r="H54" s="31" t="inlineStr">
+        <is>
+          <t>論證邏輯、立論前提與價值批判之正反比對</t>
+        </is>
+      </c>
+      <c r="I54" s="32" t="inlineStr">
+        <is>
+          <t>https://oaoadna-1313.github.io/2026-literarymeaning8lesson/23_comparison_argumentative.html</t>
+        </is>
+      </c>
+      <c r="J54" s="32" t="inlineStr">
+        <is>
+          <t>https://github.com/oaoadna-1313/2026-literarymeaning8lesson/blob/main/23_comparison_argumentative.html</t>
+        </is>
+      </c>
+      <c r="K54" s="29" t="inlineStr">
+        <is>
+          <t>✅ 100% 完成上線</t>
+        </is>
+      </c>
+      <c r="L54" s="31" t="inlineStr">
+        <is>
+          <t>雙軌切換・三色螢光筆・解題之眼・逐項剖析</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" s="26" t="n">
+        <v>51</v>
+      </c>
+      <c r="B55" s="27" t="inlineStr">
+        <is>
+          <t>第 5 課 比較篇</t>
+        </is>
+      </c>
+      <c r="C55" s="27" t="inlineStr">
+        <is>
+          <t>說明文類</t>
+        </is>
+      </c>
+      <c r="D55" s="27" t="inlineStr">
+        <is>
+          <t>24_比較篇_說明文類.html</t>
+        </is>
+      </c>
+      <c r="E55" s="27" t="inlineStr">
+        <is>
+          <t>24_comparison_expository.html</t>
+        </is>
+      </c>
+      <c r="F55" s="26" t="inlineStr">
+        <is>
+          <t>P.98 ~ P.101</t>
+        </is>
+      </c>
+      <c r="G55" s="26" t="inlineStr">
+        <is>
+          <t>8 題</t>
+        </is>
+      </c>
+      <c r="H55" s="27" t="inlineStr">
+        <is>
+          <t>自然現象、科學實驗與客觀事理數據對比</t>
+        </is>
+      </c>
+      <c r="I55" s="28" t="inlineStr">
+        <is>
+          <t>https://oaoadna-1313.github.io/2026-literarymeaning8lesson/24_comparison_expository.html</t>
+        </is>
+      </c>
+      <c r="J55" s="28" t="inlineStr">
+        <is>
+          <t>https://github.com/oaoadna-1313/2026-literarymeaning8lesson/blob/main/24_comparison_expository.html</t>
+        </is>
+      </c>
+      <c r="K55" s="29" t="inlineStr">
+        <is>
+          <t>✅ 100% 完成上線</t>
+        </is>
+      </c>
+      <c r="L55" s="27" t="inlineStr">
+        <is>
+          <t>雙軌切換・三色螢光筆・解題之眼・逐項剖析</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" s="30" t="n">
+        <v>52</v>
+      </c>
+      <c r="B56" s="31" t="inlineStr">
+        <is>
+          <t>第 5 課 比較篇</t>
+        </is>
+      </c>
+      <c r="C56" s="31" t="inlineStr">
+        <is>
+          <t>應用文類</t>
+        </is>
+      </c>
+      <c r="D56" s="31" t="inlineStr">
+        <is>
+          <t>25_比較篇_應用文類.html</t>
+        </is>
+      </c>
+      <c r="E56" s="31" t="inlineStr">
+        <is>
+          <t>25_comparison_practical.html</t>
+        </is>
+      </c>
+      <c r="F56" s="30" t="inlineStr">
+        <is>
+          <t>P.102 ~ P.105</t>
+        </is>
+      </c>
+      <c r="G56" s="30" t="inlineStr">
+        <is>
+          <t>10 題</t>
+        </is>
+      </c>
+      <c r="H56" s="31" t="inlineStr">
+        <is>
+          <t>消費方案、活動簡章、租約條款與公眾規則評比</t>
+        </is>
+      </c>
+      <c r="I56" s="32" t="inlineStr">
+        <is>
+          <t>https://oaoadna-1313.github.io/2026-literarymeaning8lesson/25_comparison_practical.html</t>
+        </is>
+      </c>
+      <c r="J56" s="32" t="inlineStr">
+        <is>
+          <t>https://github.com/oaoadna-1313/2026-literarymeaning8lesson/blob/main/25_comparison_practical.html</t>
+        </is>
+      </c>
+      <c r="K56" s="29" t="inlineStr">
+        <is>
+          <t>✅ 100% 完成上線</t>
+        </is>
+      </c>
+      <c r="L56" s="31" t="inlineStr">
+        <is>
+          <t>雙軌切換・三色螢光筆・解題之眼・逐項剖析</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" s="26" t="n">
+        <v>53</v>
+      </c>
+      <c r="B57" s="27" t="inlineStr">
+        <is>
+          <t>第 5 課 比較篇</t>
+        </is>
+      </c>
+      <c r="C57" s="27" t="inlineStr">
+        <is>
+          <t>記敘文類講義</t>
+        </is>
+      </c>
+      <c r="D57" s="27" t="inlineStr">
+        <is>
+          <t>21_比較篇_記敘文類_詳解講義.pdf</t>
+        </is>
+      </c>
+      <c r="E57" s="27" t="inlineStr">
+        <is>
+          <t>21_comparison_narrative_handout.pdf</t>
+        </is>
+      </c>
+      <c r="F57" s="26" t="inlineStr">
+        <is>
+          <t>P.88 ~ P.91</t>
+        </is>
+      </c>
+      <c r="G57" s="26" t="inlineStr">
+        <is>
+          <t>8 頁</t>
+        </is>
+      </c>
+      <c r="H57" s="27" t="inlineStr">
+        <is>
+          <t>A4單頁精編・三色螢光筆・解題之眼・語譯</t>
+        </is>
+      </c>
+      <c r="I57" s="28" t="inlineStr">
+        <is>
+          <t>https://oaoadna-1313.github.io/2026-literarymeaning8lesson/21_comparison_narrative_handout.pdf</t>
+        </is>
+      </c>
+      <c r="J57" s="28" t="inlineStr">
+        <is>
+          <t>https://github.com/oaoadna-1313/2026-literarymeaning8lesson/blob/main/21_comparison_narrative_handout.pdf</t>
+        </is>
+      </c>
+      <c r="K57" s="29" t="inlineStr">
+        <is>
+          <t>✅ 100% 完成上線</t>
+        </is>
+      </c>
+      <c r="L57" s="27" t="inlineStr">
+        <is>
+          <t>A4向量排版・一題一頁絕不溢出・精編詳解講義</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" s="30" t="n">
+        <v>54</v>
+      </c>
+      <c r="B58" s="31" t="inlineStr">
+        <is>
+          <t>第 5 課 比較篇</t>
+        </is>
+      </c>
+      <c r="C58" s="31" t="inlineStr">
+        <is>
+          <t>抒情文類講義</t>
+        </is>
+      </c>
+      <c r="D58" s="31" t="inlineStr">
+        <is>
+          <t>22_比較篇_抒情文類_詳解講義.pdf</t>
+        </is>
+      </c>
+      <c r="E58" s="31" t="inlineStr">
+        <is>
+          <t>22_comparison_lyric_handout.pdf</t>
+        </is>
+      </c>
+      <c r="F58" s="30" t="inlineStr">
+        <is>
+          <t>P.92 ~ P.94</t>
+        </is>
+      </c>
+      <c r="G58" s="30" t="inlineStr">
+        <is>
+          <t>10 頁</t>
+        </is>
+      </c>
+      <c r="H58" s="31" t="inlineStr">
+        <is>
+          <t>A4單頁精編・三色螢光筆・解題之眼・語譯</t>
+        </is>
+      </c>
+      <c r="I58" s="32" t="inlineStr">
+        <is>
+          <t>https://oaoadna-1313.github.io/2026-literarymeaning8lesson/22_comparison_lyric_handout.pdf</t>
+        </is>
+      </c>
+      <c r="J58" s="32" t="inlineStr">
+        <is>
+          <t>https://github.com/oaoadna-1313/2026-literarymeaning8lesson/blob/main/22_comparison_lyric_handout.pdf</t>
+        </is>
+      </c>
+      <c r="K58" s="29" t="inlineStr">
+        <is>
+          <t>✅ 100% 完成上線</t>
+        </is>
+      </c>
+      <c r="L58" s="31" t="inlineStr">
+        <is>
+          <t>A4向量排版・一題一頁絕不溢出・精編詳解講義</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" s="26" t="n">
+        <v>55</v>
+      </c>
+      <c r="B59" s="27" t="inlineStr">
+        <is>
+          <t>第 5 課 比較篇</t>
+        </is>
+      </c>
+      <c r="C59" s="27" t="inlineStr">
+        <is>
+          <t>議論文類講義</t>
+        </is>
+      </c>
+      <c r="D59" s="27" t="inlineStr">
+        <is>
+          <t>23_比較篇_議論文類_詳解講義.pdf</t>
+        </is>
+      </c>
+      <c r="E59" s="27" t="inlineStr">
+        <is>
+          <t>23_comparison_argumentative_handout.pdf</t>
+        </is>
+      </c>
+      <c r="F59" s="26" t="inlineStr">
+        <is>
+          <t>P.95 ~ P.97</t>
+        </is>
+      </c>
+      <c r="G59" s="26" t="inlineStr">
+        <is>
+          <t>10 頁</t>
+        </is>
+      </c>
+      <c r="H59" s="27" t="inlineStr">
+        <is>
+          <t>A4單頁精編・三色螢光筆・解題之眼・語譯</t>
+        </is>
+      </c>
+      <c r="I59" s="28" t="inlineStr">
+        <is>
+          <t>https://oaoadna-1313.github.io/2026-literarymeaning8lesson/23_comparison_argumentative_handout.pdf</t>
+        </is>
+      </c>
+      <c r="J59" s="28" t="inlineStr">
+        <is>
+          <t>https://github.com/oaoadna-1313/2026-literarymeaning8lesson/blob/main/23_comparison_argumentative_handout.pdf</t>
+        </is>
+      </c>
+      <c r="K59" s="29" t="inlineStr">
+        <is>
+          <t>✅ 100% 完成上線</t>
+        </is>
+      </c>
+      <c r="L59" s="27" t="inlineStr">
+        <is>
+          <t>A4向量排版・一題一頁絕不溢出・精編詳解講義</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" s="30" t="n">
+        <v>56</v>
+      </c>
+      <c r="B60" s="31" t="inlineStr">
+        <is>
+          <t>第 5 課 比較篇</t>
+        </is>
+      </c>
+      <c r="C60" s="31" t="inlineStr">
+        <is>
+          <t>說明文類講義</t>
+        </is>
+      </c>
+      <c r="D60" s="31" t="inlineStr">
+        <is>
+          <t>24_比較篇_說明文類_詳解講義.pdf</t>
+        </is>
+      </c>
+      <c r="E60" s="31" t="inlineStr">
+        <is>
+          <t>24_comparison_expository_handout.pdf</t>
+        </is>
+      </c>
+      <c r="F60" s="30" t="inlineStr">
+        <is>
+          <t>P.98 ~ P.101</t>
+        </is>
+      </c>
+      <c r="G60" s="30" t="inlineStr">
+        <is>
+          <t>8 頁</t>
+        </is>
+      </c>
+      <c r="H60" s="31" t="inlineStr">
+        <is>
+          <t>A4單頁精編・三色螢光筆・解題之眼・語譯</t>
+        </is>
+      </c>
+      <c r="I60" s="32" t="inlineStr">
+        <is>
+          <t>https://oaoadna-1313.github.io/2026-literarymeaning8lesson/24_comparison_expository_handout.pdf</t>
+        </is>
+      </c>
+      <c r="J60" s="32" t="inlineStr">
+        <is>
+          <t>https://github.com/oaoadna-1313/2026-literarymeaning8lesson/blob/main/24_comparison_expository_handout.pdf</t>
+        </is>
+      </c>
+      <c r="K60" s="29" t="inlineStr">
+        <is>
+          <t>✅ 100% 完成上線</t>
+        </is>
+      </c>
+      <c r="L60" s="31" t="inlineStr">
+        <is>
+          <t>A4向量排版・一題一頁絕不溢出・精編詳解講義</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" s="26" t="n">
+        <v>57</v>
+      </c>
+      <c r="B61" s="27" t="inlineStr">
+        <is>
+          <t>第 5 課 比較篇</t>
+        </is>
+      </c>
+      <c r="C61" s="27" t="inlineStr">
+        <is>
+          <t>應用文類講義</t>
+        </is>
+      </c>
+      <c r="D61" s="27" t="inlineStr">
+        <is>
+          <t>25_比較篇_應用文類_詳解講義.pdf</t>
+        </is>
+      </c>
+      <c r="E61" s="27" t="inlineStr">
+        <is>
+          <t>25_comparison_practical_handout.pdf</t>
+        </is>
+      </c>
+      <c r="F61" s="26" t="inlineStr">
+        <is>
+          <t>P.102 ~ P.105</t>
+        </is>
+      </c>
+      <c r="G61" s="26" t="inlineStr">
+        <is>
+          <t>10 頁</t>
+        </is>
+      </c>
+      <c r="H61" s="27" t="inlineStr">
+        <is>
+          <t>A4單頁精編・三色螢光筆・解題之眼・語譯</t>
+        </is>
+      </c>
+      <c r="I61" s="28" t="inlineStr">
+        <is>
+          <t>https://oaoadna-1313.github.io/2026-literarymeaning8lesson/25_comparison_practical_handout.pdf</t>
+        </is>
+      </c>
+      <c r="J61" s="28" t="inlineStr">
+        <is>
+          <t>https://github.com/oaoadna-1313/2026-literarymeaning8lesson/blob/main/25_comparison_practical_handout.pdf</t>
+        </is>
+      </c>
+      <c r="K61" s="29" t="inlineStr">
+        <is>
+          <t>✅ 100% 完成上線</t>
+        </is>
+      </c>
+      <c r="L61" s="27" t="inlineStr">
+        <is>
+          <t>A4向量排版・一題一頁絕不溢出・精編詳解講義</t>
+        </is>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" s="30" t="n">
+        <v>58</v>
+      </c>
+      <c r="B62" s="31" t="inlineStr">
+        <is>
+          <t>第 5 課 比較篇</t>
+        </is>
+      </c>
+      <c r="C62" s="31" t="inlineStr">
+        <is>
+          <t>全套合訂本講義</t>
+        </is>
+      </c>
+      <c r="D62" s="31" t="inlineStr">
+        <is>
+          <t>文意新8課_第5課比較篇_全套精編詳解講義.pdf</t>
+        </is>
+      </c>
+      <c r="E62" s="31" t="inlineStr">
+        <is>
+          <t>05_comparison_complete_handout.pdf</t>
+        </is>
+      </c>
+      <c r="F62" s="30" t="inlineStr">
+        <is>
+          <t>全書 P.88~105</t>
+        </is>
+      </c>
+      <c r="G62" s="30" t="inlineStr">
+        <is>
+          <t>48 頁</t>
+        </is>
+      </c>
+      <c r="H62" s="31" t="inlineStr">
+        <is>
+          <t>全冊大合訂本：封面+總目錄+46題單頁精編</t>
+        </is>
+      </c>
+      <c r="I62" s="32" t="inlineStr">
+        <is>
+          <t>https://oaoadna-1313.github.io/2026-literarymeaning8lesson/05_comparison_complete_handout.pdf</t>
+        </is>
+      </c>
+      <c r="J62" s="32" t="inlineStr">
+        <is>
+          <t>https://github.com/oaoadna-1313/2026-literarymeaning8lesson/blob/main/05_comparison_complete_handout.pdf</t>
+        </is>
+      </c>
+      <c r="K62" s="29" t="inlineStr">
+        <is>
+          <t>✅ 100% 完成上線</t>
+        </is>
+      </c>
+      <c r="L62" s="31" t="inlineStr">
+        <is>
+          <t>A4向量排版・一題一頁絕不溢出・精編詳解講義</t>
+        </is>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" s="26" t="n">
+        <v>59</v>
+      </c>
+      <c r="B63" s="27" t="inlineStr">
+        <is>
+          <t>第 6 課 推論篇</t>
+        </is>
+      </c>
+      <c r="C63" s="27" t="inlineStr">
+        <is>
+          <t>記敘文類</t>
+        </is>
+      </c>
+      <c r="D63" s="27" t="inlineStr">
+        <is>
+          <t>26_推論篇_記敘文類.html</t>
+        </is>
+      </c>
+      <c r="E63" s="27" t="inlineStr">
+        <is>
+          <t>26_inference_narrative.html</t>
+        </is>
+      </c>
+      <c r="F63" s="26" t="inlineStr">
+        <is>
+          <t>P.111 ~ P.113</t>
+        </is>
+      </c>
+      <c r="G63" s="26" t="inlineStr">
+        <is>
+          <t>9 題</t>
+        </is>
+      </c>
+      <c r="H63" s="27" t="inlineStr">
+        <is>
+          <t>推求事件因果、情節脈絡與言外伏筆</t>
+        </is>
+      </c>
+      <c r="I63" s="28" t="inlineStr">
+        <is>
+          <t>https://oaoadna-1313.github.io/2026-literarymeaning8lesson/26_inference_narrative.html</t>
+        </is>
+      </c>
+      <c r="J63" s="28" t="inlineStr">
+        <is>
+          <t>https://github.com/oaoadna-1313/2026-literarymeaning8lesson/blob/main/26_inference_narrative.html</t>
+        </is>
+      </c>
+      <c r="K63" s="29" t="inlineStr">
+        <is>
+          <t>✅ 100% 完成上線</t>
+        </is>
+      </c>
+      <c r="L63" s="27" t="inlineStr">
+        <is>
+          <t>雙軌切換・三色螢光筆・解題之眼・逐項剖析</t>
+        </is>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" s="30" t="n">
+        <v>60</v>
+      </c>
+      <c r="B64" s="31" t="inlineStr">
+        <is>
+          <t>第 6 課 推論篇</t>
+        </is>
+      </c>
+      <c r="C64" s="31" t="inlineStr">
+        <is>
+          <t>抒情文類</t>
+        </is>
+      </c>
+      <c r="D64" s="31" t="inlineStr">
+        <is>
+          <t>27_推論篇_抒情文類.html</t>
+        </is>
+      </c>
+      <c r="E64" s="31" t="inlineStr">
+        <is>
+          <t>27_inference_lyric.html</t>
+        </is>
+      </c>
+      <c r="F64" s="30" t="inlineStr">
+        <is>
+          <t>P.114 ~ P.116</t>
+        </is>
+      </c>
+      <c r="G64" s="30" t="inlineStr">
+        <is>
+          <t>9 題</t>
+        </is>
+      </c>
+      <c r="H64" s="31" t="inlineStr">
+        <is>
+          <t>推知心境轉折、意象寄託與生命感懷</t>
+        </is>
+      </c>
+      <c r="I64" s="32" t="inlineStr">
+        <is>
+          <t>https://oaoadna-1313.github.io/2026-literarymeaning8lesson/27_inference_lyric.html</t>
+        </is>
+      </c>
+      <c r="J64" s="32" t="inlineStr">
+        <is>
+          <t>https://github.com/oaoadna-1313/2026-literarymeaning8lesson/blob/main/27_inference_lyric.html</t>
+        </is>
+      </c>
+      <c r="K64" s="29" t="inlineStr">
+        <is>
+          <t>✅ 100% 完成上線</t>
+        </is>
+      </c>
+      <c r="L64" s="31" t="inlineStr">
+        <is>
+          <t>雙軌切換・三色螢光筆・解題之眼・逐項剖析</t>
+        </is>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" s="26" t="n">
+        <v>61</v>
+      </c>
+      <c r="B65" s="27" t="inlineStr">
+        <is>
+          <t>第 6 課 推論篇</t>
+        </is>
+      </c>
+      <c r="C65" s="27" t="inlineStr">
+        <is>
+          <t>議論文類</t>
+        </is>
+      </c>
+      <c r="D65" s="27" t="inlineStr">
+        <is>
+          <t>28_推論篇_議論文類.html</t>
+        </is>
+      </c>
+      <c r="E65" s="27" t="inlineStr">
+        <is>
+          <t>28_inference_argumentative.html</t>
+        </is>
+      </c>
+      <c r="F65" s="26" t="inlineStr">
+        <is>
+          <t>P.117 ~ P.119</t>
+        </is>
+      </c>
+      <c r="G65" s="26" t="inlineStr">
+        <is>
+          <t>10 題</t>
+        </is>
+      </c>
+      <c r="H65" s="27" t="inlineStr">
+        <is>
+          <t>推衍邏輯理路、論述前提與核心價值</t>
+        </is>
+      </c>
+      <c r="I65" s="28" t="inlineStr">
+        <is>
+          <t>https://oaoadna-1313.github.io/2026-literarymeaning8lesson/28_inference_argumentative.html</t>
+        </is>
+      </c>
+      <c r="J65" s="28" t="inlineStr">
+        <is>
+          <t>https://github.com/oaoadna-1313/2026-literarymeaning8lesson/blob/main/28_inference_argumentative.html</t>
+        </is>
+      </c>
+      <c r="K65" s="29" t="inlineStr">
+        <is>
+          <t>✅ 100% 完成上線</t>
+        </is>
+      </c>
+      <c r="L65" s="27" t="inlineStr">
+        <is>
+          <t>雙軌切換・三色螢光筆・解題之眼・逐項剖析</t>
+        </is>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" s="30" t="n">
+        <v>62</v>
+      </c>
+      <c r="B66" s="31" t="inlineStr">
+        <is>
+          <t>第 6 課 推論篇</t>
+        </is>
+      </c>
+      <c r="C66" s="31" t="inlineStr">
+        <is>
+          <t>說明文類</t>
+        </is>
+      </c>
+      <c r="D66" s="31" t="inlineStr">
+        <is>
+          <t>29_推論篇_說明文類.html</t>
+        </is>
+      </c>
+      <c r="E66" s="31" t="inlineStr">
+        <is>
+          <t>29_inference_expository.html</t>
+        </is>
+      </c>
+      <c r="F66" s="30" t="inlineStr">
+        <is>
+          <t>P.120 ~ P.122</t>
+        </is>
+      </c>
+      <c r="G66" s="30" t="inlineStr">
+        <is>
+          <t>9 題</t>
+        </is>
+      </c>
+      <c r="H66" s="31" t="inlineStr">
+        <is>
+          <t>推斷科學機理、客觀定律與未知結論</t>
+        </is>
+      </c>
+      <c r="I66" s="32" t="inlineStr">
+        <is>
+          <t>https://oaoadna-1313.github.io/2026-literarymeaning8lesson/29_inference_expository.html</t>
+        </is>
+      </c>
+      <c r="J66" s="32" t="inlineStr">
+        <is>
+          <t>https://github.com/oaoadna-1313/2026-literarymeaning8lesson/blob/main/29_inference_expository.html</t>
+        </is>
+      </c>
+      <c r="K66" s="29" t="inlineStr">
+        <is>
+          <t>✅ 100% 完成上線</t>
+        </is>
+      </c>
+      <c r="L66" s="31" t="inlineStr">
+        <is>
+          <t>雙軌切換・三色螢光筆・解題之眼・逐項剖析</t>
+        </is>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" s="26" t="n">
+        <v>63</v>
+      </c>
+      <c r="B67" s="27" t="inlineStr">
+        <is>
+          <t>第 6 課 推論篇</t>
+        </is>
+      </c>
+      <c r="C67" s="27" t="inlineStr">
+        <is>
+          <t>應用文類</t>
+        </is>
+      </c>
+      <c r="D67" s="27" t="inlineStr">
+        <is>
+          <t>30_推論篇_應用文類.html</t>
+        </is>
+      </c>
+      <c r="E67" s="27" t="inlineStr">
+        <is>
+          <t>30_inference_practical.html</t>
+        </is>
+      </c>
+      <c r="F67" s="26" t="inlineStr">
+        <is>
+          <t>P.123 ~ P.125</t>
+        </is>
+      </c>
+      <c r="G67" s="26" t="inlineStr">
+        <is>
+          <t>8 題</t>
+        </is>
+      </c>
+      <c r="H67" s="27" t="inlineStr">
+        <is>
+          <t>推敲情境用意、生活規範與實用決策</t>
+        </is>
+      </c>
+      <c r="I67" s="28" t="inlineStr">
+        <is>
+          <t>https://oaoadna-1313.github.io/2026-literarymeaning8lesson/30_inference_practical.html</t>
+        </is>
+      </c>
+      <c r="J67" s="28" t="inlineStr">
+        <is>
+          <t>https://github.com/oaoadna-1313/2026-literarymeaning8lesson/blob/main/30_inference_practical.html</t>
+        </is>
+      </c>
+      <c r="K67" s="29" t="inlineStr">
+        <is>
+          <t>✅ 100% 完成上線</t>
+        </is>
+      </c>
+      <c r="L67" s="27" t="inlineStr">
+        <is>
+          <t>雙軌切換・三色螢光筆・解題之眼・逐項剖析</t>
+        </is>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" s="30" t="n">
+        <v>64</v>
+      </c>
+      <c r="B68" s="31" t="inlineStr">
+        <is>
+          <t>第 6 課 推論篇</t>
+        </is>
+      </c>
+      <c r="C68" s="31" t="inlineStr">
+        <is>
+          <t>記敘文類講義</t>
+        </is>
+      </c>
+      <c r="D68" s="31" t="inlineStr">
+        <is>
+          <t>26_推論篇_記敘文類_詳解講義.pdf</t>
+        </is>
+      </c>
+      <c r="E68" s="31" t="inlineStr">
+        <is>
+          <t>26_inference_narrative_handout.pdf</t>
+        </is>
+      </c>
+      <c r="F68" s="30" t="inlineStr">
+        <is>
+          <t>P.111 ~ P.113</t>
+        </is>
+      </c>
+      <c r="G68" s="30" t="inlineStr">
+        <is>
+          <t>9 頁</t>
+        </is>
+      </c>
+      <c r="H68" s="31" t="inlineStr">
+        <is>
+          <t>A4單頁精編・三色螢光筆・解題之眼・語譯</t>
+        </is>
+      </c>
+      <c r="I68" s="32" t="inlineStr">
+        <is>
+          <t>https://oaoadna-1313.github.io/2026-literarymeaning8lesson/26_inference_narrative_handout.pdf</t>
+        </is>
+      </c>
+      <c r="J68" s="32" t="inlineStr">
+        <is>
+          <t>https://github.com/oaoadna-1313/2026-literarymeaning8lesson/blob/main/26_inference_narrative_handout.pdf</t>
+        </is>
+      </c>
+      <c r="K68" s="29" t="inlineStr">
+        <is>
+          <t>✅ 100% 完成上線</t>
+        </is>
+      </c>
+      <c r="L68" s="31" t="inlineStr">
+        <is>
+          <t>A4向量排版・一題一頁絕不溢出・精編詳解講義</t>
+        </is>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" s="26" t="n">
+        <v>65</v>
+      </c>
+      <c r="B69" s="27" t="inlineStr">
+        <is>
+          <t>第 6 課 推論篇</t>
+        </is>
+      </c>
+      <c r="C69" s="27" t="inlineStr">
+        <is>
+          <t>抒情文類講義</t>
+        </is>
+      </c>
+      <c r="D69" s="27" t="inlineStr">
+        <is>
+          <t>27_推論篇_抒情文類_詳解講義.pdf</t>
+        </is>
+      </c>
+      <c r="E69" s="27" t="inlineStr">
+        <is>
+          <t>27_inference_lyric_handout.pdf</t>
+        </is>
+      </c>
+      <c r="F69" s="26" t="inlineStr">
+        <is>
+          <t>P.114 ~ P.116</t>
+        </is>
+      </c>
+      <c r="G69" s="26" t="inlineStr">
+        <is>
+          <t>9 頁</t>
+        </is>
+      </c>
+      <c r="H69" s="27" t="inlineStr">
+        <is>
+          <t>A4單頁精編・三色螢光筆・解題之眼・語譯</t>
+        </is>
+      </c>
+      <c r="I69" s="28" t="inlineStr">
+        <is>
+          <t>https://oaoadna-1313.github.io/2026-literarymeaning8lesson/27_inference_lyric_handout.pdf</t>
+        </is>
+      </c>
+      <c r="J69" s="28" t="inlineStr">
+        <is>
+          <t>https://github.com/oaoadna-1313/2026-literarymeaning8lesson/blob/main/27_inference_lyric_handout.pdf</t>
+        </is>
+      </c>
+      <c r="K69" s="29" t="inlineStr">
+        <is>
+          <t>✅ 100% 完成上線</t>
+        </is>
+      </c>
+      <c r="L69" s="27" t="inlineStr">
+        <is>
+          <t>A4向量排版・一題一頁絕不溢出・精編詳解講義</t>
+        </is>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" s="30" t="n">
+        <v>66</v>
+      </c>
+      <c r="B70" s="31" t="inlineStr">
+        <is>
+          <t>第 6 課 推論篇</t>
+        </is>
+      </c>
+      <c r="C70" s="31" t="inlineStr">
+        <is>
+          <t>議論文類講義</t>
+        </is>
+      </c>
+      <c r="D70" s="31" t="inlineStr">
+        <is>
+          <t>28_推論篇_議論文類_詳解講義.pdf</t>
+        </is>
+      </c>
+      <c r="E70" s="31" t="inlineStr">
+        <is>
+          <t>28_inference_argumentative_handout.pdf</t>
+        </is>
+      </c>
+      <c r="F70" s="30" t="inlineStr">
+        <is>
+          <t>P.117 ~ P.119</t>
+        </is>
+      </c>
+      <c r="G70" s="30" t="inlineStr">
+        <is>
+          <t>10 頁</t>
+        </is>
+      </c>
+      <c r="H70" s="31" t="inlineStr">
+        <is>
+          <t>A4單頁精編・三色螢光筆・解題之眼・語譯</t>
+        </is>
+      </c>
+      <c r="I70" s="32" t="inlineStr">
+        <is>
+          <t>https://oaoadna-1313.github.io/2026-literarymeaning8lesson/28_inference_argumentative_handout.pdf</t>
+        </is>
+      </c>
+      <c r="J70" s="32" t="inlineStr">
+        <is>
+          <t>https://github.com/oaoadna-1313/2026-literarymeaning8lesson/blob/main/28_inference_argumentative_handout.pdf</t>
+        </is>
+      </c>
+      <c r="K70" s="29" t="inlineStr">
+        <is>
+          <t>✅ 100% 完成上線</t>
+        </is>
+      </c>
+      <c r="L70" s="31" t="inlineStr">
+        <is>
+          <t>A4向量排版・一題一頁絕不溢出・精編詳解講義</t>
+        </is>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" s="26" t="n">
+        <v>67</v>
+      </c>
+      <c r="B71" s="27" t="inlineStr">
+        <is>
+          <t>第 6 課 推論篇</t>
+        </is>
+      </c>
+      <c r="C71" s="27" t="inlineStr">
+        <is>
+          <t>說明文類講義</t>
+        </is>
+      </c>
+      <c r="D71" s="27" t="inlineStr">
+        <is>
+          <t>29_推論篇_說明文類_詳解講義.pdf</t>
+        </is>
+      </c>
+      <c r="E71" s="27" t="inlineStr">
+        <is>
+          <t>29_inference_expository_handout.pdf</t>
+        </is>
+      </c>
+      <c r="F71" s="26" t="inlineStr">
+        <is>
+          <t>P.120 ~ P.122</t>
+        </is>
+      </c>
+      <c r="G71" s="26" t="inlineStr">
+        <is>
+          <t>9 頁</t>
+        </is>
+      </c>
+      <c r="H71" s="27" t="inlineStr">
+        <is>
+          <t>A4單頁精編・三色螢光筆・解題之眼・語譯</t>
+        </is>
+      </c>
+      <c r="I71" s="28" t="inlineStr">
+        <is>
+          <t>https://oaoadna-1313.github.io/2026-literarymeaning8lesson/29_inference_expository_handout.pdf</t>
+        </is>
+      </c>
+      <c r="J71" s="28" t="inlineStr">
+        <is>
+          <t>https://github.com/oaoadna-1313/2026-literarymeaning8lesson/blob/main/29_inference_expository_handout.pdf</t>
+        </is>
+      </c>
+      <c r="K71" s="29" t="inlineStr">
+        <is>
+          <t>✅ 100% 完成上線</t>
+        </is>
+      </c>
+      <c r="L71" s="27" t="inlineStr">
+        <is>
+          <t>A4向量排版・一題一頁絕不溢出・精編詳解講義</t>
+        </is>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" s="30" t="n">
+        <v>68</v>
+      </c>
+      <c r="B72" s="31" t="inlineStr">
+        <is>
+          <t>第 6 課 推論篇</t>
+        </is>
+      </c>
+      <c r="C72" s="31" t="inlineStr">
+        <is>
+          <t>應用文類講義</t>
+        </is>
+      </c>
+      <c r="D72" s="31" t="inlineStr">
+        <is>
+          <t>30_推論篇_應用文類_詳解講義.pdf</t>
+        </is>
+      </c>
+      <c r="E72" s="31" t="inlineStr">
+        <is>
+          <t>30_inference_practical_handout.pdf</t>
+        </is>
+      </c>
+      <c r="F72" s="30" t="inlineStr">
+        <is>
+          <t>P.123 ~ P.125</t>
+        </is>
+      </c>
+      <c r="G72" s="30" t="inlineStr">
+        <is>
+          <t>8 頁</t>
+        </is>
+      </c>
+      <c r="H72" s="31" t="inlineStr">
+        <is>
+          <t>A4單頁精編・三色螢光筆・解題之眼・語譯</t>
+        </is>
+      </c>
+      <c r="I72" s="32" t="inlineStr">
+        <is>
+          <t>https://oaoadna-1313.github.io/2026-literarymeaning8lesson/30_inference_practical_handout.pdf</t>
+        </is>
+      </c>
+      <c r="J72" s="32" t="inlineStr">
+        <is>
+          <t>https://github.com/oaoadna-1313/2026-literarymeaning8lesson/blob/main/30_inference_practical_handout.pdf</t>
+        </is>
+      </c>
+      <c r="K72" s="29" t="inlineStr">
+        <is>
+          <t>✅ 100% 完成上線</t>
+        </is>
+      </c>
+      <c r="L72" s="31" t="inlineStr">
+        <is>
+          <t>A4向量排版・一題一頁絕不溢出・精編詳解講義</t>
+        </is>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" s="26" t="n">
+        <v>69</v>
+      </c>
+      <c r="B73" s="27" t="inlineStr">
+        <is>
+          <t>第 6 課 推論篇</t>
+        </is>
+      </c>
+      <c r="C73" s="27" t="inlineStr">
+        <is>
+          <t>全套合訂本講義</t>
+        </is>
+      </c>
+      <c r="D73" s="27" t="inlineStr">
+        <is>
+          <t>文意新8課_第6課推論篇_全套精編詳解講義.pdf</t>
+        </is>
+      </c>
+      <c r="E73" s="27" t="inlineStr">
+        <is>
+          <t>06_inference_complete_handout.pdf</t>
+        </is>
+      </c>
+      <c r="F73" s="26" t="inlineStr">
+        <is>
+          <t>全書 P.111~125</t>
+        </is>
+      </c>
+      <c r="G73" s="26" t="inlineStr">
+        <is>
+          <t>47 頁</t>
+        </is>
+      </c>
+      <c r="H73" s="27" t="inlineStr">
+        <is>
+          <t>全冊大合訂本：封面+總目錄+45題單頁精編</t>
+        </is>
+      </c>
+      <c r="I73" s="28" t="inlineStr">
+        <is>
+          <t>https://oaoadna-1313.github.io/2026-literarymeaning8lesson/06_inference_complete_handout.pdf</t>
+        </is>
+      </c>
+      <c r="J73" s="28" t="inlineStr">
+        <is>
+          <t>https://github.com/oaoadna-1313/2026-literarymeaning8lesson/blob/main/06_inference_complete_handout.pdf</t>
+        </is>
+      </c>
+      <c r="K73" s="29" t="inlineStr">
+        <is>
+          <t>✅ 100% 完成上線</t>
+        </is>
+      </c>
+      <c r="L73" s="27" t="inlineStr">
+        <is>
+          <t>A4向量排版・一題一頁絕不溢出・精編詳解講義</t>
+        </is>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" s="30" t="n">
+        <v>70</v>
+      </c>
+      <c r="B74" s="31" t="inlineStr">
+        <is>
+          <t>第 7 課 寫作手法篇</t>
+        </is>
+      </c>
+      <c r="C74" s="31" t="inlineStr">
+        <is>
+          <t>記敘文類</t>
+        </is>
+      </c>
+      <c r="D74" s="31" t="inlineStr">
+        <is>
+          <t>31_寫作手法篇_記敘文類.html</t>
+        </is>
+      </c>
+      <c r="E74" s="31" t="inlineStr">
+        <is>
+          <t>31_technique_narrative.html</t>
+        </is>
+      </c>
+      <c r="F74" s="30" t="inlineStr">
+        <is>
+          <t>P.131 ~ P.133</t>
+        </is>
+      </c>
+      <c r="G74" s="30" t="inlineStr">
+        <is>
+          <t>8 題</t>
+        </is>
+      </c>
+      <c r="H74" s="31" t="inlineStr">
+        <is>
+          <t>記敘文寫作手法：時空倒敘、插敘伏筆與視角轉換</t>
+        </is>
+      </c>
+      <c r="I74" s="32" t="inlineStr">
+        <is>
+          <t>https://oaoadna-1313.github.io/2026-literarymeaning8lesson/31_technique_narrative.html</t>
+        </is>
+      </c>
+      <c r="J74" s="32" t="inlineStr">
+        <is>
+          <t>https://github.com/oaoadna-1313/2026-literarymeaning8lesson/blob/main/31_technique_narrative.html</t>
+        </is>
+      </c>
+      <c r="K74" s="29" t="inlineStr">
+        <is>
+          <t>✅ 100% 完成上線</t>
+        </is>
+      </c>
+      <c r="L74" s="31" t="inlineStr">
+        <is>
+          <t>雙軌切換・三色螢光筆・解題之眼・逐項剖析</t>
+        </is>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" s="26" t="n">
+        <v>71</v>
+      </c>
+      <c r="B75" s="27" t="inlineStr">
+        <is>
+          <t>第 7 課 寫作手法篇</t>
+        </is>
+      </c>
+      <c r="C75" s="27" t="inlineStr">
+        <is>
+          <t>抒情文類</t>
+        </is>
+      </c>
+      <c r="D75" s="27" t="inlineStr">
+        <is>
+          <t>32_寫作手法篇_抒情文類.html</t>
+        </is>
+      </c>
+      <c r="E75" s="27" t="inlineStr">
+        <is>
+          <t>32_technique_lyric.html</t>
+        </is>
+      </c>
+      <c r="F75" s="26" t="inlineStr">
+        <is>
+          <t>P.134 ~ P.136</t>
+        </is>
+      </c>
+      <c r="G75" s="26" t="inlineStr">
+        <is>
+          <t>9 題</t>
+        </is>
+      </c>
+      <c r="H75" s="27" t="inlineStr">
+        <is>
+          <t>抒情文寫作手法：觸景生情、借物抒懷與情景交融</t>
+        </is>
+      </c>
+      <c r="I75" s="28" t="inlineStr">
+        <is>
+          <t>https://oaoadna-1313.github.io/2026-literarymeaning8lesson/32_technique_lyric.html</t>
+        </is>
+      </c>
+      <c r="J75" s="28" t="inlineStr">
+        <is>
+          <t>https://github.com/oaoadna-1313/2026-literarymeaning8lesson/blob/main/32_technique_lyric.html</t>
+        </is>
+      </c>
+      <c r="K75" s="29" t="inlineStr">
+        <is>
+          <t>✅ 100% 完成上線</t>
+        </is>
+      </c>
+      <c r="L75" s="27" t="inlineStr">
+        <is>
+          <t>雙軌切換・三色螢光筆・解題之眼・逐項剖析</t>
+        </is>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" s="30" t="n">
+        <v>72</v>
+      </c>
+      <c r="B76" s="31" t="inlineStr">
+        <is>
+          <t>第 7 課 寫作手法篇</t>
+        </is>
+      </c>
+      <c r="C76" s="31" t="inlineStr">
+        <is>
+          <t>議論文類</t>
+        </is>
+      </c>
+      <c r="D76" s="31" t="inlineStr">
+        <is>
+          <t>33_寫作手法篇_議論文類.html</t>
+        </is>
+      </c>
+      <c r="E76" s="31" t="inlineStr">
+        <is>
+          <t>33_technique_argumentative.html</t>
+        </is>
+      </c>
+      <c r="F76" s="30" t="inlineStr">
+        <is>
+          <t>P.137 ~ P.139</t>
+        </is>
+      </c>
+      <c r="G76" s="30" t="inlineStr">
+        <is>
+          <t>10 題</t>
+        </is>
+      </c>
+      <c r="H76" s="31" t="inlineStr">
+        <is>
+          <t>議論文寫作手法：破題立論、正反論證與引經據典</t>
+        </is>
+      </c>
+      <c r="I76" s="32" t="inlineStr">
+        <is>
+          <t>https://oaoadna-1313.github.io/2026-literarymeaning8lesson/33_technique_argumentative.html</t>
+        </is>
+      </c>
+      <c r="J76" s="32" t="inlineStr">
+        <is>
+          <t>https://github.com/oaoadna-1313/2026-literarymeaning8lesson/blob/main/33_technique_argumentative.html</t>
+        </is>
+      </c>
+      <c r="K76" s="29" t="inlineStr">
+        <is>
+          <t>✅ 100% 完成上線</t>
+        </is>
+      </c>
+      <c r="L76" s="31" t="inlineStr">
+        <is>
+          <t>雙軌切換・三色螢光筆・解題之眼・逐項剖析</t>
+        </is>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" s="26" t="n">
+        <v>73</v>
+      </c>
+      <c r="B77" s="27" t="inlineStr">
+        <is>
+          <t>第 7 課 寫作手法篇</t>
+        </is>
+      </c>
+      <c r="C77" s="27" t="inlineStr">
+        <is>
+          <t>說明文類</t>
+        </is>
+      </c>
+      <c r="D77" s="27" t="inlineStr">
+        <is>
+          <t>34_寫作手法篇_說明文類.html</t>
+        </is>
+      </c>
+      <c r="E77" s="27" t="inlineStr">
+        <is>
+          <t>34_technique_expository.html</t>
+        </is>
+      </c>
+      <c r="F77" s="26" t="inlineStr">
+        <is>
+          <t>P.140 ~ P.142</t>
+        </is>
+      </c>
+      <c r="G77" s="26" t="inlineStr">
+        <is>
+          <t>8 題</t>
+        </is>
+      </c>
+      <c r="H77" s="27" t="inlineStr">
+        <is>
+          <t>說明文寫作手法：分類比較、定義舉例與圖表輔助</t>
+        </is>
+      </c>
+      <c r="I77" s="28" t="inlineStr">
+        <is>
+          <t>https://oaoadna-1313.github.io/2026-literarymeaning8lesson/34_technique_expository.html</t>
+        </is>
+      </c>
+      <c r="J77" s="28" t="inlineStr">
+        <is>
+          <t>https://github.com/oaoadna-1313/2026-literarymeaning8lesson/blob/main/34_technique_expository.html</t>
+        </is>
+      </c>
+      <c r="K77" s="29" t="inlineStr">
+        <is>
+          <t>✅ 100% 完成上線</t>
+        </is>
+      </c>
+      <c r="L77" s="27" t="inlineStr">
+        <is>
+          <t>雙軌切換・三色螢光筆・解題之眼・逐項剖析</t>
+        </is>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" s="30" t="n">
+        <v>74</v>
+      </c>
+      <c r="B78" s="31" t="inlineStr">
+        <is>
+          <t>第 7 課 寫作手法篇</t>
+        </is>
+      </c>
+      <c r="C78" s="31" t="inlineStr">
+        <is>
+          <t>應用文類</t>
+        </is>
+      </c>
+      <c r="D78" s="31" t="inlineStr">
+        <is>
+          <t>35_寫作手法篇_應用文類.html</t>
+        </is>
+      </c>
+      <c r="E78" s="31" t="inlineStr">
+        <is>
+          <t>35_technique_practical.html</t>
+        </is>
+      </c>
+      <c r="F78" s="30" t="inlineStr">
+        <is>
+          <t>P.143 ~ P.145</t>
+        </is>
+      </c>
+      <c r="G78" s="30" t="inlineStr">
+        <is>
+          <t>8 題</t>
+        </is>
+      </c>
+      <c r="H78" s="31" t="inlineStr">
+        <is>
+          <t>應用文寫作手法：單據啟事、宣導規章與標語修辭</t>
+        </is>
+      </c>
+      <c r="I78" s="32" t="inlineStr">
+        <is>
+          <t>https://oaoadna-1313.github.io/2026-literarymeaning8lesson/35_technique_practical.html</t>
+        </is>
+      </c>
+      <c r="J78" s="32" t="inlineStr">
+        <is>
+          <t>https://github.com/oaoadna-1313/2026-literarymeaning8lesson/blob/main/35_technique_practical.html</t>
+        </is>
+      </c>
+      <c r="K78" s="29" t="inlineStr">
+        <is>
+          <t>✅ 100% 完成上線</t>
+        </is>
+      </c>
+      <c r="L78" s="31" t="inlineStr">
+        <is>
+          <t>雙軌切換・三色螢光筆・解題之眼・逐項剖析</t>
+        </is>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" s="26" t="n">
+        <v>75</v>
+      </c>
+      <c r="B79" s="27" t="inlineStr">
+        <is>
+          <t>第 7 課 寫作手法篇</t>
+        </is>
+      </c>
+      <c r="C79" s="27" t="inlineStr">
+        <is>
+          <t>記敘文類講義</t>
+        </is>
+      </c>
+      <c r="D79" s="27" t="inlineStr">
+        <is>
+          <t>31_寫作手法篇_記敘文類_詳解講義.pdf</t>
+        </is>
+      </c>
+      <c r="E79" s="27" t="inlineStr">
+        <is>
+          <t>31_technique_narrative_handout.pdf</t>
+        </is>
+      </c>
+      <c r="F79" s="26" t="inlineStr">
+        <is>
+          <t>P.131 ~ P.133</t>
+        </is>
+      </c>
+      <c r="G79" s="26" t="inlineStr">
+        <is>
+          <t>8 頁</t>
+        </is>
+      </c>
+      <c r="H79" s="27" t="inlineStr">
+        <is>
+          <t>A4單頁精編・三色螢光筆・解題之眼・語譯</t>
+        </is>
+      </c>
+      <c r="I79" s="28" t="inlineStr">
+        <is>
+          <t>https://oaoadna-1313.github.io/2026-literarymeaning8lesson/31_technique_narrative_handout.pdf</t>
+        </is>
+      </c>
+      <c r="J79" s="28" t="inlineStr">
+        <is>
+          <t>https://github.com/oaoadna-1313/2026-literarymeaning8lesson/blob/main/31_technique_narrative_handout.pdf</t>
+        </is>
+      </c>
+      <c r="K79" s="29" t="inlineStr">
+        <is>
+          <t>✅ 100% 完成上線</t>
+        </is>
+      </c>
+      <c r="L79" s="27" t="inlineStr">
+        <is>
+          <t>A4向量排版・一題一頁絕不溢出・精編詳解講義</t>
+        </is>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" s="30" t="n">
+        <v>76</v>
+      </c>
+      <c r="B80" s="31" t="inlineStr">
+        <is>
+          <t>第 7 課 寫作手法篇</t>
+        </is>
+      </c>
+      <c r="C80" s="31" t="inlineStr">
+        <is>
+          <t>抒情文類講義</t>
+        </is>
+      </c>
+      <c r="D80" s="31" t="inlineStr">
+        <is>
+          <t>32_寫作手法篇_抒情文類_詳解講義.pdf</t>
+        </is>
+      </c>
+      <c r="E80" s="31" t="inlineStr">
+        <is>
+          <t>32_technique_lyric_handout.pdf</t>
+        </is>
+      </c>
+      <c r="F80" s="30" t="inlineStr">
+        <is>
+          <t>P.134 ~ P.136</t>
+        </is>
+      </c>
+      <c r="G80" s="30" t="inlineStr">
+        <is>
+          <t>9 頁</t>
+        </is>
+      </c>
+      <c r="H80" s="31" t="inlineStr">
+        <is>
+          <t>A4單頁精編・三色螢光筆・解題之眼・語譯</t>
+        </is>
+      </c>
+      <c r="I80" s="32" t="inlineStr">
+        <is>
+          <t>https://oaoadna-1313.github.io/2026-literarymeaning8lesson/32_technique_lyric_handout.pdf</t>
+        </is>
+      </c>
+      <c r="J80" s="32" t="inlineStr">
+        <is>
+          <t>https://github.com/oaoadna-1313/2026-literarymeaning8lesson/blob/main/32_technique_lyric_handout.pdf</t>
+        </is>
+      </c>
+      <c r="K80" s="29" t="inlineStr">
+        <is>
+          <t>✅ 100% 完成上線</t>
+        </is>
+      </c>
+      <c r="L80" s="31" t="inlineStr">
+        <is>
+          <t>A4向量排版・一題一頁絕不溢出・精編詳解講義</t>
+        </is>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81" s="26" t="n">
+        <v>77</v>
+      </c>
+      <c r="B81" s="27" t="inlineStr">
+        <is>
+          <t>第 7 課 寫作手法篇</t>
+        </is>
+      </c>
+      <c r="C81" s="27" t="inlineStr">
+        <is>
+          <t>議論文類講義</t>
+        </is>
+      </c>
+      <c r="D81" s="27" t="inlineStr">
+        <is>
+          <t>33_寫作手法篇_議論文類_詳解講義.pdf</t>
+        </is>
+      </c>
+      <c r="E81" s="27" t="inlineStr">
+        <is>
+          <t>33_technique_argumentative_handout.pdf</t>
+        </is>
+      </c>
+      <c r="F81" s="26" t="inlineStr">
+        <is>
+          <t>P.137 ~ P.139</t>
+        </is>
+      </c>
+      <c r="G81" s="26" t="inlineStr">
+        <is>
+          <t>10 頁</t>
+        </is>
+      </c>
+      <c r="H81" s="27" t="inlineStr">
+        <is>
+          <t>A4單頁精編・三色螢光筆・解題之眼・語譯</t>
+        </is>
+      </c>
+      <c r="I81" s="28" t="inlineStr">
+        <is>
+          <t>https://oaoadna-1313.github.io/2026-literarymeaning8lesson/33_technique_argumentative_handout.pdf</t>
+        </is>
+      </c>
+      <c r="J81" s="28" t="inlineStr">
+        <is>
+          <t>https://github.com/oaoadna-1313/2026-literarymeaning8lesson/blob/main/33_technique_argumentative_handout.pdf</t>
+        </is>
+      </c>
+      <c r="K81" s="29" t="inlineStr">
+        <is>
+          <t>✅ 100% 完成上線</t>
+        </is>
+      </c>
+      <c r="L81" s="27" t="inlineStr">
+        <is>
+          <t>A4向量排版・一題一頁絕不溢出・精編詳解講義</t>
+        </is>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82" s="30" t="n">
+        <v>78</v>
+      </c>
+      <c r="B82" s="31" t="inlineStr">
+        <is>
+          <t>第 7 課 寫作手法篇</t>
+        </is>
+      </c>
+      <c r="C82" s="31" t="inlineStr">
+        <is>
+          <t>說明文類講義</t>
+        </is>
+      </c>
+      <c r="D82" s="31" t="inlineStr">
+        <is>
+          <t>34_寫作手法篇_說明文類_詳解講義.pdf</t>
+        </is>
+      </c>
+      <c r="E82" s="31" t="inlineStr">
+        <is>
+          <t>34_technique_expository_handout.pdf</t>
+        </is>
+      </c>
+      <c r="F82" s="30" t="inlineStr">
+        <is>
+          <t>P.140 ~ P.142</t>
+        </is>
+      </c>
+      <c r="G82" s="30" t="inlineStr">
+        <is>
+          <t>8 頁</t>
+        </is>
+      </c>
+      <c r="H82" s="31" t="inlineStr">
+        <is>
+          <t>A4單頁精編・三色螢光筆・解題之眼・語譯</t>
+        </is>
+      </c>
+      <c r="I82" s="32" t="inlineStr">
+        <is>
+          <t>https://oaoadna-1313.github.io/2026-literarymeaning8lesson/34_technique_expository_handout.pdf</t>
+        </is>
+      </c>
+      <c r="J82" s="32" t="inlineStr">
+        <is>
+          <t>https://github.com/oaoadna-1313/2026-literarymeaning8lesson/blob/main/34_technique_expository_handout.pdf</t>
+        </is>
+      </c>
+      <c r="K82" s="29" t="inlineStr">
+        <is>
+          <t>✅ 100% 完成上線</t>
+        </is>
+      </c>
+      <c r="L82" s="31" t="inlineStr">
+        <is>
+          <t>A4向量排版・一題一頁絕不溢出・精編詳解講義</t>
+        </is>
+      </c>
+    </row>
+    <row r="83">
+      <c r="A83" s="26" t="n">
+        <v>79</v>
+      </c>
+      <c r="B83" s="27" t="inlineStr">
+        <is>
+          <t>第 7 課 寫作手法篇</t>
+        </is>
+      </c>
+      <c r="C83" s="27" t="inlineStr">
+        <is>
+          <t>應用文類講義</t>
+        </is>
+      </c>
+      <c r="D83" s="27" t="inlineStr">
+        <is>
+          <t>35_寫作手法篇_應用文類_詳解講義.pdf</t>
+        </is>
+      </c>
+      <c r="E83" s="27" t="inlineStr">
+        <is>
+          <t>35_technique_practical_handout.pdf</t>
+        </is>
+      </c>
+      <c r="F83" s="26" t="inlineStr">
+        <is>
+          <t>P.143 ~ P.145</t>
+        </is>
+      </c>
+      <c r="G83" s="26" t="inlineStr">
+        <is>
+          <t>8 頁</t>
+        </is>
+      </c>
+      <c r="H83" s="27" t="inlineStr">
+        <is>
+          <t>A4單頁精編・三色螢光筆・解題之眼・語譯</t>
+        </is>
+      </c>
+      <c r="I83" s="28" t="inlineStr">
+        <is>
+          <t>https://oaoadna-1313.github.io/2026-literarymeaning8lesson/35_technique_practical_handout.pdf</t>
+        </is>
+      </c>
+      <c r="J83" s="28" t="inlineStr">
+        <is>
+          <t>https://github.com/oaoadna-1313/2026-literarymeaning8lesson/blob/main/35_technique_practical_handout.pdf</t>
+        </is>
+      </c>
+      <c r="K83" s="29" t="inlineStr">
+        <is>
+          <t>✅ 100% 完成上線</t>
+        </is>
+      </c>
+      <c r="L83" s="27" t="inlineStr">
+        <is>
+          <t>A4向量排版・一題一頁絕不溢出・精編詳解講義</t>
+        </is>
+      </c>
+    </row>
+    <row r="84">
+      <c r="A84" s="30" t="n">
+        <v>80</v>
+      </c>
+      <c r="B84" s="31" t="inlineStr">
+        <is>
+          <t>第 7 課 寫作手法篇</t>
+        </is>
+      </c>
+      <c r="C84" s="31" t="inlineStr">
+        <is>
+          <t>全套合訂本講義</t>
+        </is>
+      </c>
+      <c r="D84" s="31" t="inlineStr">
+        <is>
+          <t>文意新8課_第7課寫作手法篇_全套精編詳解講義.pdf</t>
+        </is>
+      </c>
+      <c r="E84" s="31" t="inlineStr">
+        <is>
+          <t>07_technique_complete_handout.pdf</t>
+        </is>
+      </c>
+      <c r="F84" s="30" t="inlineStr">
+        <is>
+          <t>全書 P.131~145</t>
+        </is>
+      </c>
+      <c r="G84" s="30" t="inlineStr">
+        <is>
+          <t>45 頁</t>
+        </is>
+      </c>
+      <c r="H84" s="31" t="inlineStr">
+        <is>
+          <t>全冊大合訂本：封面+總目錄+43題單頁精編</t>
+        </is>
+      </c>
+      <c r="I84" s="32" t="inlineStr">
+        <is>
+          <t>https://oaoadna-1313.github.io/2026-literarymeaning8lesson/07_technique_complete_handout.pdf</t>
+        </is>
+      </c>
+      <c r="J84" s="32" t="inlineStr">
+        <is>
+          <t>https://github.com/oaoadna-1313/2026-literarymeaning8lesson/blob/main/07_technique_complete_handout.pdf</t>
+        </is>
+      </c>
+      <c r="K84" s="29" t="inlineStr">
+        <is>
+          <t>✅ 100% 完成上線</t>
+        </is>
+      </c>
+      <c r="L84" s="31" t="inlineStr">
+        <is>
+          <t>A4向量排版・一題一頁絕不溢出・精編詳解講義</t>
+        </is>
+      </c>
+    </row>
+    <row r="85">
+      <c r="A85" s="26" t="n">
+        <v>81</v>
+      </c>
+      <c r="B85" s="27" t="inlineStr">
+        <is>
+          <t>第 8 課 圖表判讀篇</t>
+        </is>
+      </c>
+      <c r="C85" s="27" t="inlineStr">
+        <is>
+          <t>說明文類</t>
+        </is>
+      </c>
+      <c r="D85" s="27" t="inlineStr">
+        <is>
+          <t>36_圖表判讀篇_說明文類.html</t>
+        </is>
+      </c>
+      <c r="E85" s="27" t="inlineStr">
+        <is>
+          <t>36_diagram_expository.html</t>
+        </is>
+      </c>
+      <c r="F85" s="26" t="inlineStr">
+        <is>
+          <t>P.150 ~ P.155</t>
+        </is>
+      </c>
+      <c r="G85" s="26" t="inlineStr">
+        <is>
+          <t>10 題</t>
+        </is>
+      </c>
+      <c r="H85" s="27" t="inlineStr">
+        <is>
+          <t>統計圖表剖析：折線長條趨勢、圓餅占比與地圖路徑</t>
+        </is>
+      </c>
+      <c r="I85" s="28" t="inlineStr">
+        <is>
+          <t>https://oaoadna-1313.github.io/2026-literarymeaning8lesson/36_diagram_expository.html</t>
+        </is>
+      </c>
+      <c r="J85" s="28" t="inlineStr">
+        <is>
+          <t>https://github.com/oaoadna-1313/2026-literarymeaning8lesson/blob/main/36_diagram_expository.html</t>
+        </is>
+      </c>
+      <c r="K85" s="29" t="inlineStr">
+        <is>
+          <t>✅ 100% 完成上線</t>
+        </is>
+      </c>
+      <c r="L85" s="27" t="inlineStr">
+        <is>
+          <t>雙軌切換・三色螢光筆・解題之眼・逐項剖析</t>
+        </is>
+      </c>
+    </row>
+    <row r="86">
+      <c r="A86" s="30" t="n">
+        <v>82</v>
+      </c>
+      <c r="B86" s="31" t="inlineStr">
+        <is>
+          <t>第 8 課 圖表判讀篇</t>
+        </is>
+      </c>
+      <c r="C86" s="31" t="inlineStr">
+        <is>
+          <t>應用文類</t>
+        </is>
+      </c>
+      <c r="D86" s="31" t="inlineStr">
+        <is>
+          <t>37_圖表判讀篇_應用文類.html</t>
+        </is>
+      </c>
+      <c r="E86" s="31" t="inlineStr">
+        <is>
+          <t>37_diagram_practical.html</t>
+        </is>
+      </c>
+      <c r="F86" s="30" t="inlineStr">
+        <is>
+          <t>P.156 ~ P.160</t>
+        </is>
+      </c>
+      <c r="G86" s="30" t="inlineStr">
+        <is>
+          <t>10 題</t>
+        </is>
+      </c>
+      <c r="H86" s="31" t="inlineStr">
+        <is>
+          <t>實用圖文辨讀：公共海報規章、金字塔指南與資訊APP</t>
+        </is>
+      </c>
+      <c r="I86" s="32" t="inlineStr">
+        <is>
+          <t>https://oaoadna-1313.github.io/2026-literarymeaning8lesson/37_diagram_practical.html</t>
+        </is>
+      </c>
+      <c r="J86" s="32" t="inlineStr">
+        <is>
+          <t>https://github.com/oaoadna-1313/2026-literarymeaning8lesson/blob/main/37_diagram_practical.html</t>
+        </is>
+      </c>
+      <c r="K86" s="29" t="inlineStr">
+        <is>
+          <t>✅ 100% 完成上線</t>
+        </is>
+      </c>
+      <c r="L86" s="31" t="inlineStr">
+        <is>
+          <t>雙軌切換・三色螢光筆・解題之眼・逐項剖析</t>
+        </is>
+      </c>
+    </row>
+    <row r="87">
+      <c r="A87" s="26" t="n">
+        <v>83</v>
+      </c>
+      <c r="B87" s="27" t="inlineStr">
+        <is>
+          <t>第 8 課 圖表判讀篇</t>
+        </is>
+      </c>
+      <c r="C87" s="27" t="inlineStr">
+        <is>
+          <t>說明文類講義</t>
+        </is>
+      </c>
+      <c r="D87" s="27" t="inlineStr">
+        <is>
+          <t>36_圖表判讀篇_說明文類_詳解講義.pdf</t>
+        </is>
+      </c>
+      <c r="E87" s="27" t="inlineStr">
+        <is>
+          <t>36_diagram_expository_handout.pdf</t>
+        </is>
+      </c>
+      <c r="F87" s="26" t="inlineStr">
+        <is>
+          <t>P.150 ~ P.155</t>
+        </is>
+      </c>
+      <c r="G87" s="26" t="inlineStr">
+        <is>
+          <t>10 頁</t>
+        </is>
+      </c>
+      <c r="H87" s="27" t="inlineStr">
+        <is>
+          <t>A4單頁精編・全彩高清圖表・解題之眼</t>
+        </is>
+      </c>
+      <c r="I87" s="28" t="inlineStr">
+        <is>
+          <t>https://oaoadna-1313.github.io/2026-literarymeaning8lesson/36_diagram_expository_handout.pdf</t>
+        </is>
+      </c>
+      <c r="J87" s="28" t="inlineStr">
+        <is>
+          <t>https://github.com/oaoadna-1313/2026-literarymeaning8lesson/blob/main/36_diagram_expository_handout.pdf</t>
+        </is>
+      </c>
+      <c r="K87" s="29" t="inlineStr">
+        <is>
+          <t>✅ 100% 完成上線</t>
+        </is>
+      </c>
+      <c r="L87" s="27" t="inlineStr">
+        <is>
+          <t>A4向量排版・一題一頁絕不溢出・精編詳解講義</t>
+        </is>
+      </c>
+    </row>
+    <row r="88">
+      <c r="A88" s="30" t="n">
+        <v>84</v>
+      </c>
+      <c r="B88" s="31" t="inlineStr">
+        <is>
+          <t>第 8 課 圖表判讀篇</t>
+        </is>
+      </c>
+      <c r="C88" s="31" t="inlineStr">
+        <is>
+          <t>應用文類講義</t>
+        </is>
+      </c>
+      <c r="D88" s="31" t="inlineStr">
+        <is>
+          <t>37_圖表判讀篇_應用文類_詳解講義.pdf</t>
+        </is>
+      </c>
+      <c r="E88" s="31" t="inlineStr">
+        <is>
+          <t>37_diagram_practical_handout.pdf</t>
+        </is>
+      </c>
+      <c r="F88" s="30" t="inlineStr">
+        <is>
+          <t>P.156 ~ P.160</t>
+        </is>
+      </c>
+      <c r="G88" s="30" t="inlineStr">
+        <is>
+          <t>10 頁</t>
+        </is>
+      </c>
+      <c r="H88" s="31" t="inlineStr">
+        <is>
+          <t>A4單頁精編・全彩高清圖表・解題之眼</t>
+        </is>
+      </c>
+      <c r="I88" s="32" t="inlineStr">
+        <is>
+          <t>https://oaoadna-1313.github.io/2026-literarymeaning8lesson/37_diagram_practical_handout.pdf</t>
+        </is>
+      </c>
+      <c r="J88" s="32" t="inlineStr">
+        <is>
+          <t>https://github.com/oaoadna-1313/2026-literarymeaning8lesson/blob/main/37_diagram_practical_handout.pdf</t>
+        </is>
+      </c>
+      <c r="K88" s="29" t="inlineStr">
+        <is>
+          <t>✅ 100% 完成上線</t>
+        </is>
+      </c>
+      <c r="L88" s="31" t="inlineStr">
+        <is>
+          <t>A4向量排版・一題一頁絕不溢出・精編詳解講義</t>
+        </is>
+      </c>
+    </row>
+    <row r="89">
+      <c r="A89" s="26" t="n">
+        <v>85</v>
+      </c>
+      <c r="B89" s="27" t="inlineStr">
+        <is>
+          <t>第 8 課 圖表判讀篇</t>
+        </is>
+      </c>
+      <c r="C89" s="27" t="inlineStr">
+        <is>
+          <t>全套合訂本講義</t>
+        </is>
+      </c>
+      <c r="D89" s="27" t="inlineStr">
+        <is>
+          <t>文意新8課_第8課圖表判讀篇_全套精編詳解講義.pdf</t>
+        </is>
+      </c>
+      <c r="E89" s="27" t="inlineStr">
+        <is>
+          <t>08_diagram_complete_handout.pdf</t>
+        </is>
+      </c>
+      <c r="F89" s="26" t="inlineStr">
+        <is>
+          <t>全書 P.150~160</t>
+        </is>
+      </c>
+      <c r="G89" s="26" t="inlineStr">
+        <is>
+          <t>22 頁</t>
+        </is>
+      </c>
+      <c r="H89" s="27" t="inlineStr">
+        <is>
+          <t>全冊大合訂本：封面+總目錄+20題單頁精編</t>
+        </is>
+      </c>
+      <c r="I89" s="28" t="inlineStr">
+        <is>
+          <t>https://oaoadna-1313.github.io/2026-literarymeaning8lesson/08_diagram_complete_handout.pdf</t>
+        </is>
+      </c>
+      <c r="J89" s="28" t="inlineStr">
+        <is>
+          <t>https://github.com/oaoadna-1313/2026-literarymeaning8lesson/blob/main/08_diagram_complete_handout.pdf</t>
+        </is>
+      </c>
+      <c r="K89" s="29" t="inlineStr">
+        <is>
+          <t>✅ 100% 完成上線</t>
+        </is>
+      </c>
+      <c r="L89" s="27" t="inlineStr">
+        <is>
+          <t>A4向量排版・一題一頁絕不溢出・精編詳解講義</t>
+        </is>
+      </c>
+    </row>
+    <row r="90">
+      <c r="A90" s="30" t="n">
+        <v>86</v>
+      </c>
+      <c r="B90" s="31" t="inlineStr">
+        <is>
+          <t>成果驗收（一）</t>
+        </is>
+      </c>
+      <c r="C90" s="31" t="inlineStr">
+        <is>
+          <t>全冊綜合評量(一)</t>
+        </is>
+      </c>
+      <c r="D90" s="31" t="inlineStr">
+        <is>
+          <t>38_成果驗收(一).html</t>
+        </is>
+      </c>
+      <c r="E90" s="31" t="inlineStr">
+        <is>
+          <t>38_review_assessment_1.html</t>
+        </is>
+      </c>
+      <c r="F90" s="30" t="inlineStr">
+        <is>
+          <t>P.162 ~ P.167</t>
+        </is>
+      </c>
+      <c r="G90" s="30" t="inlineStr">
+        <is>
+          <t>20 題</t>
+        </is>
+      </c>
+      <c r="H90" s="31" t="inlineStr">
+        <is>
+          <t>全冊綜合評量（一）：古典文言、記敘抒情、議論說明與生活圖表</t>
+        </is>
+      </c>
+      <c r="I90" s="32" t="inlineStr">
+        <is>
+          <t>https://oaoadna-1313.github.io/2026-literarymeaning8lesson/38_review_assessment_1.html</t>
+        </is>
+      </c>
+      <c r="J90" s="32" t="inlineStr">
+        <is>
+          <t>https://github.com/oaoadna-1313/2026-literarymeaning8lesson/blob/main/38_review_assessment_1.html</t>
+        </is>
+      </c>
+      <c r="K90" s="29" t="inlineStr">
+        <is>
+          <t>✅ 100% 完成上線</t>
+        </is>
+      </c>
+      <c r="L90" s="31" t="inlineStr">
+        <is>
+          <t>雙軌切換・三色螢光筆・解題之眼・全彩圖表・即時核對</t>
+        </is>
+      </c>
+    </row>
+    <row r="91">
+      <c r="A91" s="26" t="n">
+        <v>87</v>
+      </c>
+      <c r="B91" s="27" t="inlineStr">
+        <is>
+          <t>成果驗收（一）講義</t>
+        </is>
+      </c>
+      <c r="C91" s="27" t="inlineStr">
+        <is>
+          <t>詳解講義(PDF)</t>
+        </is>
+      </c>
+      <c r="D91" s="27" t="inlineStr">
+        <is>
+          <t>38_成果驗收(一)_詳解講義.pdf</t>
+        </is>
+      </c>
+      <c r="E91" s="27" t="inlineStr">
+        <is>
+          <t>38_review_assessment_1_handout.pdf</t>
+        </is>
+      </c>
+      <c r="F91" s="26" t="inlineStr">
+        <is>
+          <t>P.162 ~ P.167</t>
+        </is>
+      </c>
+      <c r="G91" s="26" t="inlineStr">
+        <is>
+          <t>20 頁</t>
+        </is>
+      </c>
+      <c r="H91" s="27" t="inlineStr">
+        <is>
+          <t>A4向量排版・一題一頁絕不溢出・三色螢光筆・解題之眼・語譯</t>
+        </is>
+      </c>
+      <c r="I91" s="28" t="inlineStr">
+        <is>
+          <t>https://oaoadna-1313.github.io/2026-literarymeaning8lesson/38_review_assessment_1_handout.pdf</t>
+        </is>
+      </c>
+      <c r="J91" s="28" t="inlineStr">
+        <is>
+          <t>https://github.com/oaoadna-1313/2026-literarymeaning8lesson/blob/main/38_review_assessment_1_handout.pdf</t>
+        </is>
+      </c>
+      <c r="K91" s="29" t="inlineStr">
+        <is>
+          <t>✅ 100% 完成上線</t>
+        </is>
+      </c>
+      <c r="L91" s="27" t="inlineStr">
+        <is>
+          <t>A4向量排版・一題一頁絕不溢出・精編詳解講義</t>
+        </is>
+      </c>
+    </row>
+    <row r="92">
+      <c r="A92" s="30" t="n">
+        <v>88</v>
+      </c>
+      <c r="B92" s="31" t="inlineStr">
+        <is>
+          <t>成果驗收（二）</t>
+        </is>
+      </c>
+      <c r="C92" s="31" t="inlineStr">
+        <is>
+          <t>全冊綜合評量(二)</t>
+        </is>
+      </c>
+      <c r="D92" s="31" t="inlineStr">
+        <is>
+          <t>39_成果驗收(二).html</t>
+        </is>
+      </c>
+      <c r="E92" s="31" t="inlineStr">
+        <is>
+          <t>39_review_assessment_2.html</t>
+        </is>
+      </c>
+      <c r="F92" s="30" t="inlineStr">
+        <is>
+          <t>P.168 ~ P.176</t>
+        </is>
+      </c>
+      <c r="G92" s="30" t="inlineStr">
+        <is>
+          <t>19 題</t>
+        </is>
+      </c>
+      <c r="H92" s="31" t="inlineStr">
+        <is>
+          <t>全冊綜合評量（二）：哲理寓言、跨領域科普、公共海報與多元對讀</t>
+        </is>
+      </c>
+      <c r="I92" s="32" t="inlineStr">
+        <is>
+          <t>https://oaoadna-1313.github.io/2026-literarymeaning8lesson/39_review_assessment_2.html</t>
+        </is>
+      </c>
+      <c r="J92" s="32" t="inlineStr">
+        <is>
+          <t>https://github.com/oaoadna-1313/2026-literarymeaning8lesson/blob/main/39_review_assessment_2.html</t>
+        </is>
+      </c>
+      <c r="K92" s="29" t="inlineStr">
+        <is>
+          <t>✅ 100% 完成上線</t>
+        </is>
+      </c>
+      <c r="L92" s="31" t="inlineStr">
+        <is>
+          <t>雙軌切換・三色螢光筆・解題之眼・全彩圖表・即時核對</t>
+        </is>
+      </c>
+    </row>
+    <row r="93">
+      <c r="A93" s="26" t="n">
+        <v>89</v>
+      </c>
+      <c r="B93" s="27" t="inlineStr">
+        <is>
+          <t>成果驗收（二）講義</t>
+        </is>
+      </c>
+      <c r="C93" s="27" t="inlineStr">
+        <is>
+          <t>詳解講義(PDF)</t>
+        </is>
+      </c>
+      <c r="D93" s="27" t="inlineStr">
+        <is>
+          <t>39_成果驗收(二)_詳解講義.pdf</t>
+        </is>
+      </c>
+      <c r="E93" s="27" t="inlineStr">
+        <is>
+          <t>39_review_assessment_2_handout.pdf</t>
+        </is>
+      </c>
+      <c r="F93" s="26" t="inlineStr">
+        <is>
+          <t>P.168 ~ P.176</t>
+        </is>
+      </c>
+      <c r="G93" s="26" t="inlineStr">
+        <is>
+          <t>19 頁</t>
+        </is>
+      </c>
+      <c r="H93" s="27" t="inlineStr">
+        <is>
+          <t>A4向量排版・一題一頁絕不溢出・三色螢光筆・解題之眼・語譯</t>
+        </is>
+      </c>
+      <c r="I93" s="28" t="inlineStr">
+        <is>
+          <t>https://oaoadna-1313.github.io/2026-literarymeaning8lesson/39_review_assessment_2_handout.pdf</t>
+        </is>
+      </c>
+      <c r="J93" s="28" t="inlineStr">
+        <is>
+          <t>https://github.com/oaoadna-1313/2026-literarymeaning8lesson/blob/main/39_review_assessment_2_handout.pdf</t>
+        </is>
+      </c>
+      <c r="K93" s="29" t="inlineStr">
+        <is>
+          <t>✅ 100% 完成上線</t>
+        </is>
+      </c>
+      <c r="L93" s="27" t="inlineStr">
+        <is>
+          <t>A4向量排版・一題一頁絕不溢出・精編詳解講義</t>
+        </is>
+      </c>
+    </row>
+    <row r="94">
+      <c r="A94" s="30" t="n">
+        <v>90</v>
+      </c>
+      <c r="B94" s="31" t="inlineStr">
+        <is>
+          <t>成果驗收篇</t>
+        </is>
+      </c>
+      <c r="C94" s="31" t="inlineStr">
+        <is>
+          <t>全套合訂本講義(PDF)</t>
+        </is>
+      </c>
+      <c r="D94" s="31" t="inlineStr">
+        <is>
+          <t>文意新8課_成果驗收_全套精編詳解講義.pdf</t>
+        </is>
+      </c>
+      <c r="E94" s="31" t="inlineStr">
+        <is>
+          <t>09_review_complete_handout.pdf</t>
+        </is>
+      </c>
+      <c r="F94" s="30" t="inlineStr">
+        <is>
+          <t>全書 P.162~176</t>
+        </is>
+      </c>
+      <c r="G94" s="30" t="inlineStr">
+        <is>
+          <t>41 頁</t>
+        </is>
+      </c>
+      <c r="H94" s="31" t="inlineStr">
+        <is>
+          <t>全冊大合訂本：全彩封面+總目錄導覽+39題單頁精編詳解</t>
+        </is>
+      </c>
+      <c r="I94" s="32" t="inlineStr">
+        <is>
+          <t>https://oaoadna-1313.github.io/2026-literarymeaning8lesson/09_review_complete_handout.pdf</t>
+        </is>
+      </c>
+      <c r="J94" s="32" t="inlineStr">
+        <is>
+          <t>https://github.com/oaoadna-1313/2026-literarymeaning8lesson/blob/main/09_review_complete_handout.pdf</t>
+        </is>
+      </c>
+      <c r="K94" s="29" t="inlineStr">
+        <is>
+          <t>✅ 100% 完成上線</t>
+        </is>
+      </c>
+      <c r="L94" s="31" t="inlineStr">
+        <is>
+          <t>全冊大合訂本：封面+總目錄+39題單頁精編</t>
         </is>
       </c>
     </row>

</xml_diff>